<commit_message>
fix: Excel proje yükleme akışını is_critical/dashboard sütun kaldırımıyla senkronla
project_tasks.is_critical/dashboard_visible/dashboard_order kolonları düşürülürken
import-project-excel/export-project-excel edge fonksiyonları ve statik proje
şablonu güncellenmemişti; her Excel yüklemesinde görev satırları artık var
olmayan kolonlara yazmaya çalışıp sessizce başarısız oluyordu. Her iki edge
fonksiyon ve şablon (v7) bu üç alandan temizlendi, redeploy edildi.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/excel/fons-solar-proje-sablonu.xlsx
+++ b/public/excel/fons-solar-proje-sablonu.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="156">
   <si>
     <t xml:space="preserve">  FONS SOLAR   |   PROJE BİLGİLERİ</t>
   </si>
@@ -124,12 +124,6 @@
     <t>★  Yıldızlı (*) alanlar zorunludur  |  Tarih: GG.AA.YYYY  |  Bu sayfa projects tablosuna aktarılır</t>
   </si>
   <si>
-    <t xml:space="preserve">  FONS SOLAR   |   İŞ KALEMLERİ</t>
-  </si>
-  <si>
-    <t>Adım 2 — Görev listesi · Kategori · Tarih · Durum · Hedef Miktar · Kritik Yol  →  Supabase: project_tasks</t>
-  </si>
-  <si>
     <t xml:space="preserve">Görev
 Kodu</t>
   </si>
@@ -179,18 +173,6 @@
   <si>
     <t xml:space="preserve">Hedef
 Miktar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dashboard
-Göster</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dashboard
-Sıra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kritik
-mi?</t>
   </si>
   <si>
     <t xml:space="preserve">  FONS SOLAR   |   KATEGORİ AĞIRLIKLARI</t>
@@ -446,7 +428,7 @@
     <t xml:space="preserve">  FONS SOLAR   |   KULLANIM KILAVUZU</t>
   </si>
   <si>
-    <t>Şablon v6 — Sistem import yapısına birebir hizalı (14.07.2026 sadeleştirmesi)</t>
+    <t>Şablon v7 (03.08.2026: İş Kalemleri'nden Dashboard Göster/Sıra ve Kritik mi? kolonları kaldırıldı)</t>
   </si>
   <si>
     <t>1️⃣</t>
@@ -464,7 +446,7 @@
     <t>İş Kalemleri → project_tasks</t>
   </si>
   <si>
-    <t>Kategori/Durum dropdown. Süre otomatik. İlerleme % girilmez — günlük raporlardan hesaplanır. Birim/Hedef Miktar dolu olan satırlar sahadan ölçülebilir ilerleme kalemi olur; Dashboard Göster=Evet ise proje panosunda görünür. Kritik mi?=Evet işaretlenen görevler Kritik Yol listesinde çıkar.</t>
+    <t>Kategori/Durum dropdown. Birim+Hedef Miktar doldurulursa gorev sahadan gunluk raporla miktar bazli takip edilir, bos birakilirsa Durum kolonuyla takip edilir.</t>
   </si>
   <si>
     <t>3️⃣</t>
@@ -1490,14 +1472,10 @@
     <col min="13" max="13" width="26" customWidth="1"/>
     <col min="14" max="14" width="10" customWidth="1"/>
     <col min="15" max="15" width="12" customWidth="1"/>
-    <col min="16" max="16" width="13" customWidth="1"/>
-    <col min="17" max="17" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>34</v>
-      </c>
+      <c r="A1" s="1"/>
       <c r="B1"/>
       <c r="C1"/>
       <c r="D1"/>
@@ -1517,9 +1495,7 @@
       <c r="R1"/>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>35</v>
-      </c>
+      <c r="A2" s="2"/>
       <c r="B2"/>
       <c r="C2"/>
       <c r="D2"/>
@@ -1540,58 +1516,49 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>41</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="I4" s="9" t="s">
         <v>11</v>
       </c>
       <c r="J4" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="L4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="M4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="N4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="O4" s="9" t="s">
         <v>47</v>
-      </c>
-      <c r="N4" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="O4" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="P4" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q4" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="R4" s="9" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -1613,9 +1580,6 @@
       <c r="M5" s="10"/>
       <c r="N5" s="10"/>
       <c r="O5" s="10"/>
-      <c r="P5" s="10"/>
-      <c r="Q5" s="10"/>
-      <c r="R5" s="10"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="10"/>
@@ -1636,9 +1600,6 @@
       <c r="M6" s="10"/>
       <c r="N6" s="10"/>
       <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="10"/>
@@ -1659,9 +1620,6 @@
       <c r="M7" s="10"/>
       <c r="N7" s="10"/>
       <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="10"/>
-      <c r="R7" s="10"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
@@ -1682,9 +1640,6 @@
       <c r="M8" s="10"/>
       <c r="N8" s="10"/>
       <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
@@ -1705,9 +1660,6 @@
       <c r="M9" s="10"/>
       <c r="N9" s="10"/>
       <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="10"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
@@ -1728,9 +1680,6 @@
       <c r="M10" s="10"/>
       <c r="N10" s="10"/>
       <c r="O10" s="10"/>
-      <c r="P10" s="10"/>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="10"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
@@ -1751,9 +1700,6 @@
       <c r="M11" s="10"/>
       <c r="N11" s="10"/>
       <c r="O11" s="10"/>
-      <c r="P11" s="10"/>
-      <c r="Q11" s="10"/>
-      <c r="R11" s="10"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
@@ -1774,9 +1720,6 @@
       <c r="M12" s="10"/>
       <c r="N12" s="10"/>
       <c r="O12" s="10"/>
-      <c r="P12" s="10"/>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="10"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
@@ -1797,9 +1740,6 @@
       <c r="M13" s="10"/>
       <c r="N13" s="10"/>
       <c r="O13" s="10"/>
-      <c r="P13" s="10"/>
-      <c r="Q13" s="10"/>
-      <c r="R13" s="10"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
@@ -1820,9 +1760,6 @@
       <c r="M14" s="10"/>
       <c r="N14" s="10"/>
       <c r="O14" s="10"/>
-      <c r="P14" s="10"/>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
@@ -1843,9 +1780,6 @@
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
       <c r="O15" s="10"/>
-      <c r="P15" s="10"/>
-      <c r="Q15" s="10"/>
-      <c r="R15" s="10"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
@@ -1866,9 +1800,6 @@
       <c r="M16" s="10"/>
       <c r="N16" s="10"/>
       <c r="O16" s="10"/>
-      <c r="P16" s="10"/>
-      <c r="Q16" s="10"/>
-      <c r="R16" s="10"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
@@ -1889,9 +1820,6 @@
       <c r="M17" s="10"/>
       <c r="N17" s="10"/>
       <c r="O17" s="10"/>
-      <c r="P17" s="10"/>
-      <c r="Q17" s="10"/>
-      <c r="R17" s="10"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="10"/>
@@ -1912,9 +1840,6 @@
       <c r="M18" s="10"/>
       <c r="N18" s="10"/>
       <c r="O18" s="10"/>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="10"/>
-      <c r="R18" s="10"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="10"/>
@@ -1935,9 +1860,6 @@
       <c r="M19" s="10"/>
       <c r="N19" s="10"/>
       <c r="O19" s="10"/>
-      <c r="P19" s="10"/>
-      <c r="Q19" s="10"/>
-      <c r="R19" s="10"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="10"/>
@@ -1958,9 +1880,6 @@
       <c r="M20" s="10"/>
       <c r="N20" s="10"/>
       <c r="O20" s="10"/>
-      <c r="P20" s="10"/>
-      <c r="Q20" s="10"/>
-      <c r="R20" s="10"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="10"/>
@@ -1981,9 +1900,6 @@
       <c r="M21" s="10"/>
       <c r="N21" s="10"/>
       <c r="O21" s="10"/>
-      <c r="P21" s="10"/>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="10"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="10"/>
@@ -2004,9 +1920,6 @@
       <c r="M22" s="10"/>
       <c r="N22" s="10"/>
       <c r="O22" s="10"/>
-      <c r="P22" s="10"/>
-      <c r="Q22" s="10"/>
-      <c r="R22" s="10"/>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="10"/>
@@ -2027,9 +1940,6 @@
       <c r="M23" s="10"/>
       <c r="N23" s="10"/>
       <c r="O23" s="10"/>
-      <c r="P23" s="10"/>
-      <c r="Q23" s="10"/>
-      <c r="R23" s="10"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="10"/>
@@ -2050,9 +1960,6 @@
       <c r="M24" s="10"/>
       <c r="N24" s="10"/>
       <c r="O24" s="10"/>
-      <c r="P24" s="10"/>
-      <c r="Q24" s="10"/>
-      <c r="R24" s="10"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="10"/>
@@ -2073,9 +1980,6 @@
       <c r="M25" s="10"/>
       <c r="N25" s="10"/>
       <c r="O25" s="10"/>
-      <c r="P25" s="10"/>
-      <c r="Q25" s="10"/>
-      <c r="R25" s="10"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
@@ -2096,9 +2000,6 @@
       <c r="M26" s="10"/>
       <c r="N26" s="10"/>
       <c r="O26" s="10"/>
-      <c r="P26" s="10"/>
-      <c r="Q26" s="10"/>
-      <c r="R26" s="10"/>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="10"/>
@@ -2119,9 +2020,6 @@
       <c r="M27" s="10"/>
       <c r="N27" s="10"/>
       <c r="O27" s="10"/>
-      <c r="P27" s="10"/>
-      <c r="Q27" s="10"/>
-      <c r="R27" s="10"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
@@ -2142,9 +2040,6 @@
       <c r="M28" s="10"/>
       <c r="N28" s="10"/>
       <c r="O28" s="10"/>
-      <c r="P28" s="10"/>
-      <c r="Q28" s="10"/>
-      <c r="R28" s="10"/>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="10"/>
@@ -2165,9 +2060,6 @@
       <c r="M29" s="10"/>
       <c r="N29" s="10"/>
       <c r="O29" s="10"/>
-      <c r="P29" s="10"/>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="10"/>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" s="10"/>
@@ -2188,9 +2080,6 @@
       <c r="M30" s="10"/>
       <c r="N30" s="10"/>
       <c r="O30" s="10"/>
-      <c r="P30" s="10"/>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
@@ -2211,9 +2100,6 @@
       <c r="M31" s="10"/>
       <c r="N31" s="10"/>
       <c r="O31" s="10"/>
-      <c r="P31" s="10"/>
-      <c r="Q31" s="10"/>
-      <c r="R31" s="10"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" s="10"/>
@@ -2234,9 +2120,6 @@
       <c r="M32" s="10"/>
       <c r="N32" s="10"/>
       <c r="O32" s="10"/>
-      <c r="P32" s="10"/>
-      <c r="Q32" s="10"/>
-      <c r="R32" s="10"/>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" s="10"/>
@@ -2257,9 +2140,6 @@
       <c r="M33" s="10"/>
       <c r="N33" s="10"/>
       <c r="O33" s="10"/>
-      <c r="P33" s="10"/>
-      <c r="Q33" s="10"/>
-      <c r="R33" s="10"/>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" s="10"/>
@@ -2280,9 +2160,6 @@
       <c r="M34" s="10"/>
       <c r="N34" s="10"/>
       <c r="O34" s="10"/>
-      <c r="P34" s="10"/>
-      <c r="Q34" s="10"/>
-      <c r="R34" s="10"/>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
@@ -2303,9 +2180,6 @@
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
       <c r="O35" s="10"/>
-      <c r="P35" s="10"/>
-      <c r="Q35" s="10"/>
-      <c r="R35" s="10"/>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
@@ -2326,9 +2200,6 @@
       <c r="M36" s="10"/>
       <c r="N36" s="10"/>
       <c r="O36" s="10"/>
-      <c r="P36" s="10"/>
-      <c r="Q36" s="10"/>
-      <c r="R36" s="10"/>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" s="10"/>
@@ -2349,9 +2220,6 @@
       <c r="M37" s="10"/>
       <c r="N37" s="10"/>
       <c r="O37" s="10"/>
-      <c r="P37" s="10"/>
-      <c r="Q37" s="10"/>
-      <c r="R37" s="10"/>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" s="10"/>
@@ -2372,9 +2240,6 @@
       <c r="M38" s="10"/>
       <c r="N38" s="10"/>
       <c r="O38" s="10"/>
-      <c r="P38" s="10"/>
-      <c r="Q38" s="10"/>
-      <c r="R38" s="10"/>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" s="10"/>
@@ -2395,9 +2260,6 @@
       <c r="M39" s="10"/>
       <c r="N39" s="10"/>
       <c r="O39" s="10"/>
-      <c r="P39" s="10"/>
-      <c r="Q39" s="10"/>
-      <c r="R39" s="10"/>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" s="10"/>
@@ -2418,9 +2280,6 @@
       <c r="M40" s="10"/>
       <c r="N40" s="10"/>
       <c r="O40" s="10"/>
-      <c r="P40" s="10"/>
-      <c r="Q40" s="10"/>
-      <c r="R40" s="10"/>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41" s="10"/>
@@ -2441,9 +2300,6 @@
       <c r="M41" s="10"/>
       <c r="N41" s="10"/>
       <c r="O41" s="10"/>
-      <c r="P41" s="10"/>
-      <c r="Q41" s="10"/>
-      <c r="R41" s="10"/>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" s="10"/>
@@ -2464,9 +2320,6 @@
       <c r="M42" s="10"/>
       <c r="N42" s="10"/>
       <c r="O42" s="10"/>
-      <c r="P42" s="10"/>
-      <c r="Q42" s="10"/>
-      <c r="R42" s="10"/>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" s="10"/>
@@ -2487,9 +2340,6 @@
       <c r="M43" s="10"/>
       <c r="N43" s="10"/>
       <c r="O43" s="10"/>
-      <c r="P43" s="10"/>
-      <c r="Q43" s="10"/>
-      <c r="R43" s="10"/>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44" s="10"/>
@@ -2510,9 +2360,6 @@
       <c r="M44" s="10"/>
       <c r="N44" s="10"/>
       <c r="O44" s="10"/>
-      <c r="P44" s="10"/>
-      <c r="Q44" s="10"/>
-      <c r="R44" s="10"/>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="10"/>
@@ -2533,9 +2380,6 @@
       <c r="M45" s="10"/>
       <c r="N45" s="10"/>
       <c r="O45" s="10"/>
-      <c r="P45" s="10"/>
-      <c r="Q45" s="10"/>
-      <c r="R45" s="10"/>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="10"/>
@@ -2556,9 +2400,6 @@
       <c r="M46" s="10"/>
       <c r="N46" s="10"/>
       <c r="O46" s="10"/>
-      <c r="P46" s="10"/>
-      <c r="Q46" s="10"/>
-      <c r="R46" s="10"/>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" s="10"/>
@@ -2579,9 +2420,6 @@
       <c r="M47" s="10"/>
       <c r="N47" s="10"/>
       <c r="O47" s="10"/>
-      <c r="P47" s="10"/>
-      <c r="Q47" s="10"/>
-      <c r="R47" s="10"/>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="10"/>
@@ -2602,9 +2440,6 @@
       <c r="M48" s="10"/>
       <c r="N48" s="10"/>
       <c r="O48" s="10"/>
-      <c r="P48" s="10"/>
-      <c r="Q48" s="10"/>
-      <c r="R48" s="10"/>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" s="10"/>
@@ -2625,9 +2460,6 @@
       <c r="M49" s="10"/>
       <c r="N49" s="10"/>
       <c r="O49" s="10"/>
-      <c r="P49" s="10"/>
-      <c r="Q49" s="10"/>
-      <c r="R49" s="10"/>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" s="10"/>
@@ -2648,9 +2480,6 @@
       <c r="M50" s="10"/>
       <c r="N50" s="10"/>
       <c r="O50" s="10"/>
-      <c r="P50" s="10"/>
-      <c r="Q50" s="10"/>
-      <c r="R50" s="10"/>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" s="10"/>
@@ -2671,9 +2500,6 @@
       <c r="M51" s="10"/>
       <c r="N51" s="10"/>
       <c r="O51" s="10"/>
-      <c r="P51" s="10"/>
-      <c r="Q51" s="10"/>
-      <c r="R51" s="10"/>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A52" s="10"/>
@@ -2694,9 +2520,6 @@
       <c r="M52" s="10"/>
       <c r="N52" s="10"/>
       <c r="O52" s="10"/>
-      <c r="P52" s="10"/>
-      <c r="Q52" s="10"/>
-      <c r="R52" s="10"/>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A53" s="10"/>
@@ -2717,9 +2540,6 @@
       <c r="M53" s="10"/>
       <c r="N53" s="10"/>
       <c r="O53" s="10"/>
-      <c r="P53" s="10"/>
-      <c r="Q53" s="10"/>
-      <c r="R53" s="10"/>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A54" s="10"/>
@@ -2740,9 +2560,6 @@
       <c r="M54" s="10"/>
       <c r="N54" s="10"/>
       <c r="O54" s="10"/>
-      <c r="P54" s="10"/>
-      <c r="Q54" s="10"/>
-      <c r="R54" s="10"/>
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A55" s="10"/>
@@ -2763,9 +2580,6 @@
       <c r="M55" s="10"/>
       <c r="N55" s="10"/>
       <c r="O55" s="10"/>
-      <c r="P55" s="10"/>
-      <c r="Q55" s="10"/>
-      <c r="R55" s="10"/>
     </row>
     <row r="56" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A56" s="10"/>
@@ -2786,9 +2600,6 @@
       <c r="M56" s="10"/>
       <c r="N56" s="10"/>
       <c r="O56" s="10"/>
-      <c r="P56" s="10"/>
-      <c r="Q56" s="10"/>
-      <c r="R56" s="10"/>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A57" s="10"/>
@@ -2809,9 +2620,6 @@
       <c r="M57" s="10"/>
       <c r="N57" s="10"/>
       <c r="O57" s="10"/>
-      <c r="P57" s="10"/>
-      <c r="Q57" s="10"/>
-      <c r="R57" s="10"/>
     </row>
     <row r="58" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A58" s="10"/>
@@ -2832,9 +2640,6 @@
       <c r="M58" s="10"/>
       <c r="N58" s="10"/>
       <c r="O58" s="10"/>
-      <c r="P58" s="10"/>
-      <c r="Q58" s="10"/>
-      <c r="R58" s="10"/>
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A59" s="10"/>
@@ -2855,9 +2660,6 @@
       <c r="M59" s="10"/>
       <c r="N59" s="10"/>
       <c r="O59" s="10"/>
-      <c r="P59" s="10"/>
-      <c r="Q59" s="10"/>
-      <c r="R59" s="10"/>
     </row>
     <row r="60" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A60" s="10"/>
@@ -2878,9 +2680,6 @@
       <c r="M60" s="10"/>
       <c r="N60" s="10"/>
       <c r="O60" s="10"/>
-      <c r="P60" s="10"/>
-      <c r="Q60" s="10"/>
-      <c r="R60" s="10"/>
     </row>
     <row r="61" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A61" s="10"/>
@@ -2901,9 +2700,6 @@
       <c r="M61" s="10"/>
       <c r="N61" s="10"/>
       <c r="O61" s="10"/>
-      <c r="P61" s="10"/>
-      <c r="Q61" s="10"/>
-      <c r="R61" s="10"/>
     </row>
     <row r="62" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A62" s="10"/>
@@ -2924,9 +2720,6 @@
       <c r="M62" s="10"/>
       <c r="N62" s="10"/>
       <c r="O62" s="10"/>
-      <c r="P62" s="10"/>
-      <c r="Q62" s="10"/>
-      <c r="R62" s="10"/>
     </row>
     <row r="63" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A63" s="10"/>
@@ -2947,9 +2740,6 @@
       <c r="M63" s="10"/>
       <c r="N63" s="10"/>
       <c r="O63" s="10"/>
-      <c r="P63" s="10"/>
-      <c r="Q63" s="10"/>
-      <c r="R63" s="10"/>
     </row>
     <row r="64" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A64" s="10"/>
@@ -2970,9 +2760,6 @@
       <c r="M64" s="10"/>
       <c r="N64" s="10"/>
       <c r="O64" s="10"/>
-      <c r="P64" s="10"/>
-      <c r="Q64" s="10"/>
-      <c r="R64" s="10"/>
     </row>
     <row r="65" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A65" s="10"/>
@@ -2993,9 +2780,6 @@
       <c r="M65" s="10"/>
       <c r="N65" s="10"/>
       <c r="O65" s="10"/>
-      <c r="P65" s="10"/>
-      <c r="Q65" s="10"/>
-      <c r="R65" s="10"/>
     </row>
     <row r="66" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A66" s="10"/>
@@ -3016,9 +2800,6 @@
       <c r="M66" s="10"/>
       <c r="N66" s="10"/>
       <c r="O66" s="10"/>
-      <c r="P66" s="10"/>
-      <c r="Q66" s="10"/>
-      <c r="R66" s="10"/>
     </row>
     <row r="67" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A67" s="10"/>
@@ -3039,9 +2820,6 @@
       <c r="M67" s="10"/>
       <c r="N67" s="10"/>
       <c r="O67" s="10"/>
-      <c r="P67" s="10"/>
-      <c r="Q67" s="10"/>
-      <c r="R67" s="10"/>
     </row>
     <row r="68" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A68" s="10"/>
@@ -3062,9 +2840,6 @@
       <c r="M68" s="10"/>
       <c r="N68" s="10"/>
       <c r="O68" s="10"/>
-      <c r="P68" s="10"/>
-      <c r="Q68" s="10"/>
-      <c r="R68" s="10"/>
     </row>
     <row r="69" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A69" s="10"/>
@@ -3085,9 +2860,6 @@
       <c r="M69" s="10"/>
       <c r="N69" s="10"/>
       <c r="O69" s="10"/>
-      <c r="P69" s="10"/>
-      <c r="Q69" s="10"/>
-      <c r="R69" s="10"/>
     </row>
     <row r="70" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A70" s="10"/>
@@ -3108,9 +2880,6 @@
       <c r="M70" s="10"/>
       <c r="N70" s="10"/>
       <c r="O70" s="10"/>
-      <c r="P70" s="10"/>
-      <c r="Q70" s="10"/>
-      <c r="R70" s="10"/>
     </row>
     <row r="71" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A71" s="10"/>
@@ -3131,9 +2900,6 @@
       <c r="M71" s="10"/>
       <c r="N71" s="10"/>
       <c r="O71" s="10"/>
-      <c r="P71" s="10"/>
-      <c r="Q71" s="10"/>
-      <c r="R71" s="10"/>
     </row>
     <row r="72" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A72" s="10"/>
@@ -3154,9 +2920,6 @@
       <c r="M72" s="10"/>
       <c r="N72" s="10"/>
       <c r="O72" s="10"/>
-      <c r="P72" s="10"/>
-      <c r="Q72" s="10"/>
-      <c r="R72" s="10"/>
     </row>
     <row r="73" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A73" s="10"/>
@@ -3177,9 +2940,6 @@
       <c r="M73" s="10"/>
       <c r="N73" s="10"/>
       <c r="O73" s="10"/>
-      <c r="P73" s="10"/>
-      <c r="Q73" s="10"/>
-      <c r="R73" s="10"/>
     </row>
     <row r="74" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A74" s="10"/>
@@ -3200,9 +2960,6 @@
       <c r="M74" s="10"/>
       <c r="N74" s="10"/>
       <c r="O74" s="10"/>
-      <c r="P74" s="10"/>
-      <c r="Q74" s="10"/>
-      <c r="R74" s="10"/>
     </row>
     <row r="75" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A75" s="10"/>
@@ -3223,9 +2980,6 @@
       <c r="M75" s="10"/>
       <c r="N75" s="10"/>
       <c r="O75" s="10"/>
-      <c r="P75" s="10"/>
-      <c r="Q75" s="10"/>
-      <c r="R75" s="10"/>
     </row>
     <row r="76" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A76" s="10"/>
@@ -3246,9 +3000,6 @@
       <c r="M76" s="10"/>
       <c r="N76" s="10"/>
       <c r="O76" s="10"/>
-      <c r="P76" s="10"/>
-      <c r="Q76" s="10"/>
-      <c r="R76" s="10"/>
     </row>
     <row r="77" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A77" s="10"/>
@@ -3269,9 +3020,6 @@
       <c r="M77" s="10"/>
       <c r="N77" s="10"/>
       <c r="O77" s="10"/>
-      <c r="P77" s="10"/>
-      <c r="Q77" s="10"/>
-      <c r="R77" s="10"/>
     </row>
     <row r="78" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A78" s="10"/>
@@ -3292,9 +3040,6 @@
       <c r="M78" s="10"/>
       <c r="N78" s="10"/>
       <c r="O78" s="10"/>
-      <c r="P78" s="10"/>
-      <c r="Q78" s="10"/>
-      <c r="R78" s="10"/>
     </row>
     <row r="79" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A79" s="10"/>
@@ -3315,9 +3060,6 @@
       <c r="M79" s="10"/>
       <c r="N79" s="10"/>
       <c r="O79" s="10"/>
-      <c r="P79" s="10"/>
-      <c r="Q79" s="10"/>
-      <c r="R79" s="10"/>
     </row>
     <row r="80" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A80" s="10"/>
@@ -3338,9 +3080,6 @@
       <c r="M80" s="10"/>
       <c r="N80" s="10"/>
       <c r="O80" s="10"/>
-      <c r="P80" s="10"/>
-      <c r="Q80" s="10"/>
-      <c r="R80" s="10"/>
     </row>
     <row r="81" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A81" s="10"/>
@@ -3361,9 +3100,6 @@
       <c r="M81" s="10"/>
       <c r="N81" s="10"/>
       <c r="O81" s="10"/>
-      <c r="P81" s="10"/>
-      <c r="Q81" s="10"/>
-      <c r="R81" s="10"/>
     </row>
     <row r="82" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A82" s="10"/>
@@ -3384,9 +3120,6 @@
       <c r="M82" s="10"/>
       <c r="N82" s="10"/>
       <c r="O82" s="10"/>
-      <c r="P82" s="10"/>
-      <c r="Q82" s="10"/>
-      <c r="R82" s="10"/>
     </row>
     <row r="83" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A83" s="10"/>
@@ -3407,9 +3140,6 @@
       <c r="M83" s="10"/>
       <c r="N83" s="10"/>
       <c r="O83" s="10"/>
-      <c r="P83" s="10"/>
-      <c r="Q83" s="10"/>
-      <c r="R83" s="10"/>
     </row>
     <row r="84" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A84" s="10"/>
@@ -3430,9 +3160,6 @@
       <c r="M84" s="10"/>
       <c r="N84" s="10"/>
       <c r="O84" s="10"/>
-      <c r="P84" s="10"/>
-      <c r="Q84" s="10"/>
-      <c r="R84" s="10"/>
     </row>
     <row r="85" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A85" s="10"/>
@@ -3453,9 +3180,6 @@
       <c r="M85" s="10"/>
       <c r="N85" s="10"/>
       <c r="O85" s="10"/>
-      <c r="P85" s="10"/>
-      <c r="Q85" s="10"/>
-      <c r="R85" s="10"/>
     </row>
     <row r="86" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A86" s="10"/>
@@ -3476,9 +3200,6 @@
       <c r="M86" s="10"/>
       <c r="N86" s="10"/>
       <c r="O86" s="10"/>
-      <c r="P86" s="10"/>
-      <c r="Q86" s="10"/>
-      <c r="R86" s="10"/>
     </row>
     <row r="87" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A87" s="10"/>
@@ -3499,9 +3220,6 @@
       <c r="M87" s="10"/>
       <c r="N87" s="10"/>
       <c r="O87" s="10"/>
-      <c r="P87" s="10"/>
-      <c r="Q87" s="10"/>
-      <c r="R87" s="10"/>
     </row>
     <row r="88" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A88" s="10"/>
@@ -3522,9 +3240,6 @@
       <c r="M88" s="10"/>
       <c r="N88" s="10"/>
       <c r="O88" s="10"/>
-      <c r="P88" s="10"/>
-      <c r="Q88" s="10"/>
-      <c r="R88" s="10"/>
     </row>
     <row r="89" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A89" s="10"/>
@@ -3545,9 +3260,6 @@
       <c r="M89" s="10"/>
       <c r="N89" s="10"/>
       <c r="O89" s="10"/>
-      <c r="P89" s="10"/>
-      <c r="Q89" s="10"/>
-      <c r="R89" s="10"/>
     </row>
     <row r="90" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A90" s="10"/>
@@ -3568,9 +3280,6 @@
       <c r="M90" s="10"/>
       <c r="N90" s="10"/>
       <c r="O90" s="10"/>
-      <c r="P90" s="10"/>
-      <c r="Q90" s="10"/>
-      <c r="R90" s="10"/>
     </row>
     <row r="91" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A91" s="10"/>
@@ -3591,9 +3300,6 @@
       <c r="M91" s="10"/>
       <c r="N91" s="10"/>
       <c r="O91" s="10"/>
-      <c r="P91" s="10"/>
-      <c r="Q91" s="10"/>
-      <c r="R91" s="10"/>
     </row>
     <row r="92" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A92" s="10"/>
@@ -3614,9 +3320,6 @@
       <c r="M92" s="10"/>
       <c r="N92" s="10"/>
       <c r="O92" s="10"/>
-      <c r="P92" s="10"/>
-      <c r="Q92" s="10"/>
-      <c r="R92" s="10"/>
     </row>
     <row r="93" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A93" s="10"/>
@@ -3637,9 +3340,6 @@
       <c r="M93" s="10"/>
       <c r="N93" s="10"/>
       <c r="O93" s="10"/>
-      <c r="P93" s="10"/>
-      <c r="Q93" s="10"/>
-      <c r="R93" s="10"/>
     </row>
     <row r="94" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A94" s="10"/>
@@ -3660,9 +3360,6 @@
       <c r="M94" s="10"/>
       <c r="N94" s="10"/>
       <c r="O94" s="10"/>
-      <c r="P94" s="10"/>
-      <c r="Q94" s="10"/>
-      <c r="R94" s="10"/>
     </row>
     <row r="95" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A95" s="10"/>
@@ -3683,9 +3380,6 @@
       <c r="M95" s="10"/>
       <c r="N95" s="10"/>
       <c r="O95" s="10"/>
-      <c r="P95" s="10"/>
-      <c r="Q95" s="10"/>
-      <c r="R95" s="10"/>
     </row>
     <row r="96" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A96" s="10"/>
@@ -3706,9 +3400,6 @@
       <c r="M96" s="10"/>
       <c r="N96" s="10"/>
       <c r="O96" s="10"/>
-      <c r="P96" s="10"/>
-      <c r="Q96" s="10"/>
-      <c r="R96" s="10"/>
     </row>
     <row r="97" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A97" s="10"/>
@@ -3729,9 +3420,6 @@
       <c r="M97" s="10"/>
       <c r="N97" s="10"/>
       <c r="O97" s="10"/>
-      <c r="P97" s="10"/>
-      <c r="Q97" s="10"/>
-      <c r="R97" s="10"/>
     </row>
     <row r="98" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A98" s="10"/>
@@ -3752,9 +3440,6 @@
       <c r="M98" s="10"/>
       <c r="N98" s="10"/>
       <c r="O98" s="10"/>
-      <c r="P98" s="10"/>
-      <c r="Q98" s="10"/>
-      <c r="R98" s="10"/>
     </row>
     <row r="99" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A99" s="10"/>
@@ -3775,9 +3460,6 @@
       <c r="M99" s="10"/>
       <c r="N99" s="10"/>
       <c r="O99" s="10"/>
-      <c r="P99" s="10"/>
-      <c r="Q99" s="10"/>
-      <c r="R99" s="10"/>
     </row>
     <row r="100" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A100" s="10"/>
@@ -3798,9 +3480,6 @@
       <c r="M100" s="10"/>
       <c r="N100" s="10"/>
       <c r="O100" s="10"/>
-      <c r="P100" s="10"/>
-      <c r="Q100" s="10"/>
-      <c r="R100" s="10"/>
     </row>
     <row r="101" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A101" s="10"/>
@@ -3821,9 +3500,6 @@
       <c r="M101" s="10"/>
       <c r="N101" s="10"/>
       <c r="O101" s="10"/>
-      <c r="P101" s="10"/>
-      <c r="Q101" s="10"/>
-      <c r="R101" s="10"/>
     </row>
     <row r="102" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A102" s="10"/>
@@ -3844,9 +3520,6 @@
       <c r="M102" s="10"/>
       <c r="N102" s="10"/>
       <c r="O102" s="10"/>
-      <c r="P102" s="10"/>
-      <c r="Q102" s="10"/>
-      <c r="R102" s="10"/>
     </row>
     <row r="103" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A103" s="10"/>
@@ -3867,9 +3540,6 @@
       <c r="M103" s="10"/>
       <c r="N103" s="10"/>
       <c r="O103" s="10"/>
-      <c r="P103" s="10"/>
-      <c r="Q103" s="10"/>
-      <c r="R103" s="10"/>
     </row>
     <row r="104" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A104" s="10"/>
@@ -3890,9 +3560,6 @@
       <c r="M104" s="10"/>
       <c r="N104" s="10"/>
       <c r="O104" s="10"/>
-      <c r="P104" s="10"/>
-      <c r="Q104" s="10"/>
-      <c r="R104" s="10"/>
     </row>
     <row r="105" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A105" s="10"/>
@@ -3913,9 +3580,6 @@
       <c r="M105" s="10"/>
       <c r="N105" s="10"/>
       <c r="O105" s="10"/>
-      <c r="P105" s="10"/>
-      <c r="Q105" s="10"/>
-      <c r="R105" s="10"/>
     </row>
     <row r="106" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A106" s="10"/>
@@ -3936,9 +3600,6 @@
       <c r="M106" s="10"/>
       <c r="N106" s="10"/>
       <c r="O106" s="10"/>
-      <c r="P106" s="10"/>
-      <c r="Q106" s="10"/>
-      <c r="R106" s="10"/>
     </row>
     <row r="107" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A107" s="10"/>
@@ -3959,9 +3620,6 @@
       <c r="M107" s="10"/>
       <c r="N107" s="10"/>
       <c r="O107" s="10"/>
-      <c r="P107" s="10"/>
-      <c r="Q107" s="10"/>
-      <c r="R107" s="10"/>
     </row>
     <row r="108" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A108" s="10"/>
@@ -3982,9 +3640,6 @@
       <c r="M108" s="10"/>
       <c r="N108" s="10"/>
       <c r="O108" s="10"/>
-      <c r="P108" s="10"/>
-      <c r="Q108" s="10"/>
-      <c r="R108" s="10"/>
     </row>
     <row r="109" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A109" s="10"/>
@@ -4005,9 +3660,6 @@
       <c r="M109" s="10"/>
       <c r="N109" s="10"/>
       <c r="O109" s="10"/>
-      <c r="P109" s="10"/>
-      <c r="Q109" s="10"/>
-      <c r="R109" s="10"/>
     </row>
     <row r="110" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A110" s="10"/>
@@ -4028,9 +3680,6 @@
       <c r="M110" s="10"/>
       <c r="N110" s="10"/>
       <c r="O110" s="10"/>
-      <c r="P110" s="10"/>
-      <c r="Q110" s="10"/>
-      <c r="R110" s="10"/>
     </row>
     <row r="111" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A111" s="10"/>
@@ -4051,9 +3700,6 @@
       <c r="M111" s="10"/>
       <c r="N111" s="10"/>
       <c r="O111" s="10"/>
-      <c r="P111" s="10"/>
-      <c r="Q111" s="10"/>
-      <c r="R111" s="10"/>
     </row>
     <row r="112" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A112" s="10"/>
@@ -4074,9 +3720,6 @@
       <c r="M112" s="10"/>
       <c r="N112" s="10"/>
       <c r="O112" s="10"/>
-      <c r="P112" s="10"/>
-      <c r="Q112" s="10"/>
-      <c r="R112" s="10"/>
     </row>
     <row r="113" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A113" s="10"/>
@@ -4097,9 +3740,6 @@
       <c r="M113" s="10"/>
       <c r="N113" s="10"/>
       <c r="O113" s="10"/>
-      <c r="P113" s="10"/>
-      <c r="Q113" s="10"/>
-      <c r="R113" s="10"/>
     </row>
     <row r="114" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A114" s="10"/>
@@ -4120,9 +3760,6 @@
       <c r="M114" s="10"/>
       <c r="N114" s="10"/>
       <c r="O114" s="10"/>
-      <c r="P114" s="10"/>
-      <c r="Q114" s="10"/>
-      <c r="R114" s="10"/>
     </row>
     <row r="115" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A115" s="10"/>
@@ -4143,9 +3780,6 @@
       <c r="M115" s="10"/>
       <c r="N115" s="10"/>
       <c r="O115" s="10"/>
-      <c r="P115" s="10"/>
-      <c r="Q115" s="10"/>
-      <c r="R115" s="10"/>
     </row>
     <row r="116" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A116" s="10"/>
@@ -4166,9 +3800,6 @@
       <c r="M116" s="10"/>
       <c r="N116" s="10"/>
       <c r="O116" s="10"/>
-      <c r="P116" s="10"/>
-      <c r="Q116" s="10"/>
-      <c r="R116" s="10"/>
     </row>
     <row r="117" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A117" s="10"/>
@@ -4189,9 +3820,6 @@
       <c r="M117" s="10"/>
       <c r="N117" s="10"/>
       <c r="O117" s="10"/>
-      <c r="P117" s="10"/>
-      <c r="Q117" s="10"/>
-      <c r="R117" s="10"/>
     </row>
     <row r="118" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A118" s="10"/>
@@ -4212,9 +3840,6 @@
       <c r="M118" s="10"/>
       <c r="N118" s="10"/>
       <c r="O118" s="10"/>
-      <c r="P118" s="10"/>
-      <c r="Q118" s="10"/>
-      <c r="R118" s="10"/>
     </row>
     <row r="119" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A119" s="10"/>
@@ -4235,9 +3860,6 @@
       <c r="M119" s="10"/>
       <c r="N119" s="10"/>
       <c r="O119" s="10"/>
-      <c r="P119" s="10"/>
-      <c r="Q119" s="10"/>
-      <c r="R119" s="10"/>
     </row>
     <row r="120" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A120" s="10"/>
@@ -4258,9 +3880,6 @@
       <c r="M120" s="10"/>
       <c r="N120" s="10"/>
       <c r="O120" s="10"/>
-      <c r="P120" s="10"/>
-      <c r="Q120" s="10"/>
-      <c r="R120" s="10"/>
     </row>
     <row r="121" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A121" s="10"/>
@@ -4281,9 +3900,6 @@
       <c r="M121" s="10"/>
       <c r="N121" s="10"/>
       <c r="O121" s="10"/>
-      <c r="P121" s="10"/>
-      <c r="Q121" s="10"/>
-      <c r="R121" s="10"/>
     </row>
     <row r="122" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A122" s="10"/>
@@ -4304,9 +3920,6 @@
       <c r="M122" s="10"/>
       <c r="N122" s="10"/>
       <c r="O122" s="10"/>
-      <c r="P122" s="10"/>
-      <c r="Q122" s="10"/>
-      <c r="R122" s="10"/>
     </row>
     <row r="123" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A123" s="10"/>
@@ -4327,9 +3940,6 @@
       <c r="M123" s="10"/>
       <c r="N123" s="10"/>
       <c r="O123" s="10"/>
-      <c r="P123" s="10"/>
-      <c r="Q123" s="10"/>
-      <c r="R123" s="10"/>
     </row>
     <row r="124" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A124" s="10"/>
@@ -4350,9 +3960,6 @@
       <c r="M124" s="10"/>
       <c r="N124" s="10"/>
       <c r="O124" s="10"/>
-      <c r="P124" s="10"/>
-      <c r="Q124" s="10"/>
-      <c r="R124" s="10"/>
     </row>
     <row r="125" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A125" s="10"/>
@@ -4373,9 +3980,6 @@
       <c r="M125" s="10"/>
       <c r="N125" s="10"/>
       <c r="O125" s="10"/>
-      <c r="P125" s="10"/>
-      <c r="Q125" s="10"/>
-      <c r="R125" s="10"/>
     </row>
     <row r="126" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A126" s="10"/>
@@ -4396,9 +4000,6 @@
       <c r="M126" s="10"/>
       <c r="N126" s="10"/>
       <c r="O126" s="10"/>
-      <c r="P126" s="10"/>
-      <c r="Q126" s="10"/>
-      <c r="R126" s="10"/>
     </row>
     <row r="127" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A127" s="10"/>
@@ -4419,9 +4020,6 @@
       <c r="M127" s="10"/>
       <c r="N127" s="10"/>
       <c r="O127" s="10"/>
-      <c r="P127" s="10"/>
-      <c r="Q127" s="10"/>
-      <c r="R127" s="10"/>
     </row>
     <row r="128" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A128" s="10"/>
@@ -4442,9 +4040,6 @@
       <c r="M128" s="10"/>
       <c r="N128" s="10"/>
       <c r="O128" s="10"/>
-      <c r="P128" s="10"/>
-      <c r="Q128" s="10"/>
-      <c r="R128" s="10"/>
     </row>
     <row r="129" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A129" s="10"/>
@@ -4465,9 +4060,6 @@
       <c r="M129" s="10"/>
       <c r="N129" s="10"/>
       <c r="O129" s="10"/>
-      <c r="P129" s="10"/>
-      <c r="Q129" s="10"/>
-      <c r="R129" s="10"/>
     </row>
     <row r="130" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A130" s="10"/>
@@ -4488,9 +4080,6 @@
       <c r="M130" s="10"/>
       <c r="N130" s="10"/>
       <c r="O130" s="10"/>
-      <c r="P130" s="10"/>
-      <c r="Q130" s="10"/>
-      <c r="R130" s="10"/>
     </row>
     <row r="131" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A131" s="10"/>
@@ -4511,9 +4100,6 @@
       <c r="M131" s="10"/>
       <c r="N131" s="10"/>
       <c r="O131" s="10"/>
-      <c r="P131" s="10"/>
-      <c r="Q131" s="10"/>
-      <c r="R131" s="10"/>
     </row>
     <row r="132" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A132" s="10"/>
@@ -4534,9 +4120,6 @@
       <c r="M132" s="10"/>
       <c r="N132" s="10"/>
       <c r="O132" s="10"/>
-      <c r="P132" s="10"/>
-      <c r="Q132" s="10"/>
-      <c r="R132" s="10"/>
     </row>
     <row r="133" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A133" s="10"/>
@@ -4557,9 +4140,6 @@
       <c r="M133" s="10"/>
       <c r="N133" s="10"/>
       <c r="O133" s="10"/>
-      <c r="P133" s="10"/>
-      <c r="Q133" s="10"/>
-      <c r="R133" s="10"/>
     </row>
     <row r="134" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A134" s="10"/>
@@ -4580,9 +4160,6 @@
       <c r="M134" s="10"/>
       <c r="N134" s="10"/>
       <c r="O134" s="10"/>
-      <c r="P134" s="10"/>
-      <c r="Q134" s="10"/>
-      <c r="R134" s="10"/>
     </row>
     <row r="135" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A135" s="10"/>
@@ -4603,9 +4180,6 @@
       <c r="M135" s="10"/>
       <c r="N135" s="10"/>
       <c r="O135" s="10"/>
-      <c r="P135" s="10"/>
-      <c r="Q135" s="10"/>
-      <c r="R135" s="10"/>
     </row>
     <row r="136" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A136" s="10"/>
@@ -4626,9 +4200,6 @@
       <c r="M136" s="10"/>
       <c r="N136" s="10"/>
       <c r="O136" s="10"/>
-      <c r="P136" s="10"/>
-      <c r="Q136" s="10"/>
-      <c r="R136" s="10"/>
     </row>
     <row r="137" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A137" s="10"/>
@@ -4649,9 +4220,6 @@
       <c r="M137" s="10"/>
       <c r="N137" s="10"/>
       <c r="O137" s="10"/>
-      <c r="P137" s="10"/>
-      <c r="Q137" s="10"/>
-      <c r="R137" s="10"/>
     </row>
     <row r="138" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A138" s="10"/>
@@ -4672,9 +4240,6 @@
       <c r="M138" s="10"/>
       <c r="N138" s="10"/>
       <c r="O138" s="10"/>
-      <c r="P138" s="10"/>
-      <c r="Q138" s="10"/>
-      <c r="R138" s="10"/>
     </row>
     <row r="139" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A139" s="10"/>
@@ -4695,9 +4260,6 @@
       <c r="M139" s="10"/>
       <c r="N139" s="10"/>
       <c r="O139" s="10"/>
-      <c r="P139" s="10"/>
-      <c r="Q139" s="10"/>
-      <c r="R139" s="10"/>
     </row>
     <row r="140" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A140" s="10"/>
@@ -4718,9 +4280,6 @@
       <c r="M140" s="10"/>
       <c r="N140" s="10"/>
       <c r="O140" s="10"/>
-      <c r="P140" s="10"/>
-      <c r="Q140" s="10"/>
-      <c r="R140" s="10"/>
     </row>
     <row r="141" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A141" s="10"/>
@@ -4741,9 +4300,6 @@
       <c r="M141" s="10"/>
       <c r="N141" s="10"/>
       <c r="O141" s="10"/>
-      <c r="P141" s="10"/>
-      <c r="Q141" s="10"/>
-      <c r="R141" s="10"/>
     </row>
     <row r="142" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A142" s="10"/>
@@ -4764,9 +4320,6 @@
       <c r="M142" s="10"/>
       <c r="N142" s="10"/>
       <c r="O142" s="10"/>
-      <c r="P142" s="10"/>
-      <c r="Q142" s="10"/>
-      <c r="R142" s="10"/>
     </row>
     <row r="143" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A143" s="10"/>
@@ -4787,9 +4340,6 @@
       <c r="M143" s="10"/>
       <c r="N143" s="10"/>
       <c r="O143" s="10"/>
-      <c r="P143" s="10"/>
-      <c r="Q143" s="10"/>
-      <c r="R143" s="10"/>
     </row>
     <row r="144" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A144" s="10"/>
@@ -4810,9 +4360,6 @@
       <c r="M144" s="10"/>
       <c r="N144" s="10"/>
       <c r="O144" s="10"/>
-      <c r="P144" s="10"/>
-      <c r="Q144" s="10"/>
-      <c r="R144" s="10"/>
     </row>
     <row r="145" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A145" s="10"/>
@@ -4833,9 +4380,6 @@
       <c r="M145" s="10"/>
       <c r="N145" s="10"/>
       <c r="O145" s="10"/>
-      <c r="P145" s="10"/>
-      <c r="Q145" s="10"/>
-      <c r="R145" s="10"/>
     </row>
     <row r="146" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A146" s="10"/>
@@ -4856,9 +4400,6 @@
       <c r="M146" s="10"/>
       <c r="N146" s="10"/>
       <c r="O146" s="10"/>
-      <c r="P146" s="10"/>
-      <c r="Q146" s="10"/>
-      <c r="R146" s="10"/>
     </row>
     <row r="147" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A147" s="10"/>
@@ -4879,9 +4420,6 @@
       <c r="M147" s="10"/>
       <c r="N147" s="10"/>
       <c r="O147" s="10"/>
-      <c r="P147" s="10"/>
-      <c r="Q147" s="10"/>
-      <c r="R147" s="10"/>
     </row>
     <row r="148" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A148" s="10"/>
@@ -4902,9 +4440,6 @@
       <c r="M148" s="10"/>
       <c r="N148" s="10"/>
       <c r="O148" s="10"/>
-      <c r="P148" s="10"/>
-      <c r="Q148" s="10"/>
-      <c r="R148" s="10"/>
     </row>
     <row r="149" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A149" s="10"/>
@@ -4925,9 +4460,6 @@
       <c r="M149" s="10"/>
       <c r="N149" s="10"/>
       <c r="O149" s="10"/>
-      <c r="P149" s="10"/>
-      <c r="Q149" s="10"/>
-      <c r="R149" s="10"/>
     </row>
     <row r="150" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A150" s="10"/>
@@ -4948,9 +4480,6 @@
       <c r="M150" s="10"/>
       <c r="N150" s="10"/>
       <c r="O150" s="10"/>
-      <c r="P150" s="10"/>
-      <c r="Q150" s="10"/>
-      <c r="R150" s="10"/>
     </row>
     <row r="151" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A151" s="10"/>
@@ -4971,9 +4500,6 @@
       <c r="M151" s="10"/>
       <c r="N151" s="10"/>
       <c r="O151" s="10"/>
-      <c r="P151" s="10"/>
-      <c r="Q151" s="10"/>
-      <c r="R151" s="10"/>
     </row>
     <row r="152" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A152" s="10"/>
@@ -4994,9 +4520,6 @@
       <c r="M152" s="10"/>
       <c r="N152" s="10"/>
       <c r="O152" s="10"/>
-      <c r="P152" s="10"/>
-      <c r="Q152" s="10"/>
-      <c r="R152" s="10"/>
     </row>
     <row r="153" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A153" s="10"/>
@@ -5017,9 +4540,6 @@
       <c r="M153" s="10"/>
       <c r="N153" s="10"/>
       <c r="O153" s="10"/>
-      <c r="P153" s="10"/>
-      <c r="Q153" s="10"/>
-      <c r="R153" s="10"/>
     </row>
     <row r="154" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A154" s="10"/>
@@ -5040,9 +4560,6 @@
       <c r="M154" s="10"/>
       <c r="N154" s="10"/>
       <c r="O154" s="10"/>
-      <c r="P154" s="10"/>
-      <c r="Q154" s="10"/>
-      <c r="R154" s="10"/>
     </row>
     <row r="155" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A155" s="10"/>
@@ -5063,9 +4580,6 @@
       <c r="M155" s="10"/>
       <c r="N155" s="10"/>
       <c r="O155" s="10"/>
-      <c r="P155" s="10"/>
-      <c r="Q155" s="10"/>
-      <c r="R155" s="10"/>
     </row>
     <row r="156" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A156" s="10"/>
@@ -5086,9 +4600,6 @@
       <c r="M156" s="10"/>
       <c r="N156" s="10"/>
       <c r="O156" s="10"/>
-      <c r="P156" s="10"/>
-      <c r="Q156" s="10"/>
-      <c r="R156" s="10"/>
     </row>
     <row r="157" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A157" s="10"/>
@@ -5109,9 +4620,6 @@
       <c r="M157" s="10"/>
       <c r="N157" s="10"/>
       <c r="O157" s="10"/>
-      <c r="P157" s="10"/>
-      <c r="Q157" s="10"/>
-      <c r="R157" s="10"/>
     </row>
     <row r="158" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A158" s="10"/>
@@ -5132,9 +4640,6 @@
       <c r="M158" s="10"/>
       <c r="N158" s="10"/>
       <c r="O158" s="10"/>
-      <c r="P158" s="10"/>
-      <c r="Q158" s="10"/>
-      <c r="R158" s="10"/>
     </row>
     <row r="159" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A159" s="10"/>
@@ -5155,9 +4660,6 @@
       <c r="M159" s="10"/>
       <c r="N159" s="10"/>
       <c r="O159" s="10"/>
-      <c r="P159" s="10"/>
-      <c r="Q159" s="10"/>
-      <c r="R159" s="10"/>
     </row>
     <row r="160" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A160" s="10"/>
@@ -5178,9 +4680,6 @@
       <c r="M160" s="10"/>
       <c r="N160" s="10"/>
       <c r="O160" s="10"/>
-      <c r="P160" s="10"/>
-      <c r="Q160" s="10"/>
-      <c r="R160" s="10"/>
     </row>
     <row r="161" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A161" s="10"/>
@@ -5201,9 +4700,6 @@
       <c r="M161" s="10"/>
       <c r="N161" s="10"/>
       <c r="O161" s="10"/>
-      <c r="P161" s="10"/>
-      <c r="Q161" s="10"/>
-      <c r="R161" s="10"/>
     </row>
     <row r="162" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A162" s="10"/>
@@ -5224,9 +4720,6 @@
       <c r="M162" s="10"/>
       <c r="N162" s="10"/>
       <c r="O162" s="10"/>
-      <c r="P162" s="10"/>
-      <c r="Q162" s="10"/>
-      <c r="R162" s="10"/>
     </row>
     <row r="163" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A163" s="10"/>
@@ -5247,9 +4740,6 @@
       <c r="M163" s="10"/>
       <c r="N163" s="10"/>
       <c r="O163" s="10"/>
-      <c r="P163" s="10"/>
-      <c r="Q163" s="10"/>
-      <c r="R163" s="10"/>
     </row>
     <row r="164" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A164" s="10"/>
@@ -5270,9 +4760,6 @@
       <c r="M164" s="10"/>
       <c r="N164" s="10"/>
       <c r="O164" s="10"/>
-      <c r="P164" s="10"/>
-      <c r="Q164" s="10"/>
-      <c r="R164" s="10"/>
     </row>
     <row r="165" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A165" s="10"/>
@@ -5293,9 +4780,6 @@
       <c r="M165" s="10"/>
       <c r="N165" s="10"/>
       <c r="O165" s="10"/>
-      <c r="P165" s="10"/>
-      <c r="Q165" s="10"/>
-      <c r="R165" s="10"/>
     </row>
     <row r="166" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A166" s="10"/>
@@ -5316,9 +4800,6 @@
       <c r="M166" s="10"/>
       <c r="N166" s="10"/>
       <c r="O166" s="10"/>
-      <c r="P166" s="10"/>
-      <c r="Q166" s="10"/>
-      <c r="R166" s="10"/>
     </row>
     <row r="167" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A167" s="10"/>
@@ -5339,9 +4820,6 @@
       <c r="M167" s="10"/>
       <c r="N167" s="10"/>
       <c r="O167" s="10"/>
-      <c r="P167" s="10"/>
-      <c r="Q167" s="10"/>
-      <c r="R167" s="10"/>
     </row>
     <row r="168" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A168" s="10"/>
@@ -5362,9 +4840,6 @@
       <c r="M168" s="10"/>
       <c r="N168" s="10"/>
       <c r="O168" s="10"/>
-      <c r="P168" s="10"/>
-      <c r="Q168" s="10"/>
-      <c r="R168" s="10"/>
     </row>
     <row r="169" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A169" s="10"/>
@@ -5385,9 +4860,6 @@
       <c r="M169" s="10"/>
       <c r="N169" s="10"/>
       <c r="O169" s="10"/>
-      <c r="P169" s="10"/>
-      <c r="Q169" s="10"/>
-      <c r="R169" s="10"/>
     </row>
     <row r="170" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A170" s="10"/>
@@ -5408,9 +4880,6 @@
       <c r="M170" s="10"/>
       <c r="N170" s="10"/>
       <c r="O170" s="10"/>
-      <c r="P170" s="10"/>
-      <c r="Q170" s="10"/>
-      <c r="R170" s="10"/>
     </row>
     <row r="171" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A171" s="10"/>
@@ -5431,9 +4900,6 @@
       <c r="M171" s="10"/>
       <c r="N171" s="10"/>
       <c r="O171" s="10"/>
-      <c r="P171" s="10"/>
-      <c r="Q171" s="10"/>
-      <c r="R171" s="10"/>
     </row>
     <row r="172" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A172" s="10"/>
@@ -5454,9 +4920,6 @@
       <c r="M172" s="10"/>
       <c r="N172" s="10"/>
       <c r="O172" s="10"/>
-      <c r="P172" s="10"/>
-      <c r="Q172" s="10"/>
-      <c r="R172" s="10"/>
     </row>
     <row r="173" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A173" s="10"/>
@@ -5477,9 +4940,6 @@
       <c r="M173" s="10"/>
       <c r="N173" s="10"/>
       <c r="O173" s="10"/>
-      <c r="P173" s="10"/>
-      <c r="Q173" s="10"/>
-      <c r="R173" s="10"/>
     </row>
     <row r="174" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A174" s="10"/>
@@ -5500,9 +4960,6 @@
       <c r="M174" s="10"/>
       <c r="N174" s="10"/>
       <c r="O174" s="10"/>
-      <c r="P174" s="10"/>
-      <c r="Q174" s="10"/>
-      <c r="R174" s="10"/>
     </row>
     <row r="175" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A175" s="10"/>
@@ -5523,9 +4980,6 @@
       <c r="M175" s="10"/>
       <c r="N175" s="10"/>
       <c r="O175" s="10"/>
-      <c r="P175" s="10"/>
-      <c r="Q175" s="10"/>
-      <c r="R175" s="10"/>
     </row>
     <row r="176" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A176" s="10"/>
@@ -5546,9 +5000,6 @@
       <c r="M176" s="10"/>
       <c r="N176" s="10"/>
       <c r="O176" s="10"/>
-      <c r="P176" s="10"/>
-      <c r="Q176" s="10"/>
-      <c r="R176" s="10"/>
     </row>
     <row r="177" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A177" s="10"/>
@@ -5569,9 +5020,6 @@
       <c r="M177" s="10"/>
       <c r="N177" s="10"/>
       <c r="O177" s="10"/>
-      <c r="P177" s="10"/>
-      <c r="Q177" s="10"/>
-      <c r="R177" s="10"/>
     </row>
     <row r="178" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A178" s="10"/>
@@ -5592,9 +5040,6 @@
       <c r="M178" s="10"/>
       <c r="N178" s="10"/>
       <c r="O178" s="10"/>
-      <c r="P178" s="10"/>
-      <c r="Q178" s="10"/>
-      <c r="R178" s="10"/>
     </row>
     <row r="179" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A179" s="10"/>
@@ -5615,9 +5060,6 @@
       <c r="M179" s="10"/>
       <c r="N179" s="10"/>
       <c r="O179" s="10"/>
-      <c r="P179" s="10"/>
-      <c r="Q179" s="10"/>
-      <c r="R179" s="10"/>
     </row>
     <row r="180" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A180" s="10"/>
@@ -5638,9 +5080,6 @@
       <c r="M180" s="10"/>
       <c r="N180" s="10"/>
       <c r="O180" s="10"/>
-      <c r="P180" s="10"/>
-      <c r="Q180" s="10"/>
-      <c r="R180" s="10"/>
     </row>
     <row r="181" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A181" s="10"/>
@@ -5661,9 +5100,6 @@
       <c r="M181" s="10"/>
       <c r="N181" s="10"/>
       <c r="O181" s="10"/>
-      <c r="P181" s="10"/>
-      <c r="Q181" s="10"/>
-      <c r="R181" s="10"/>
     </row>
     <row r="182" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A182" s="10"/>
@@ -5684,9 +5120,6 @@
       <c r="M182" s="10"/>
       <c r="N182" s="10"/>
       <c r="O182" s="10"/>
-      <c r="P182" s="10"/>
-      <c r="Q182" s="10"/>
-      <c r="R182" s="10"/>
     </row>
     <row r="183" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A183" s="10"/>
@@ -5707,9 +5140,6 @@
       <c r="M183" s="10"/>
       <c r="N183" s="10"/>
       <c r="O183" s="10"/>
-      <c r="P183" s="10"/>
-      <c r="Q183" s="10"/>
-      <c r="R183" s="10"/>
     </row>
     <row r="184" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A184" s="10"/>
@@ -5730,9 +5160,6 @@
       <c r="M184" s="10"/>
       <c r="N184" s="10"/>
       <c r="O184" s="10"/>
-      <c r="P184" s="10"/>
-      <c r="Q184" s="10"/>
-      <c r="R184" s="10"/>
     </row>
     <row r="185" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A185" s="10"/>
@@ -5753,9 +5180,6 @@
       <c r="M185" s="10"/>
       <c r="N185" s="10"/>
       <c r="O185" s="10"/>
-      <c r="P185" s="10"/>
-      <c r="Q185" s="10"/>
-      <c r="R185" s="10"/>
     </row>
     <row r="186" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A186" s="10"/>
@@ -5776,9 +5200,6 @@
       <c r="M186" s="10"/>
       <c r="N186" s="10"/>
       <c r="O186" s="10"/>
-      <c r="P186" s="10"/>
-      <c r="Q186" s="10"/>
-      <c r="R186" s="10"/>
     </row>
     <row r="187" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A187" s="10"/>
@@ -5799,9 +5220,6 @@
       <c r="M187" s="10"/>
       <c r="N187" s="10"/>
       <c r="O187" s="10"/>
-      <c r="P187" s="10"/>
-      <c r="Q187" s="10"/>
-      <c r="R187" s="10"/>
     </row>
     <row r="188" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A188" s="10"/>
@@ -5822,9 +5240,6 @@
       <c r="M188" s="10"/>
       <c r="N188" s="10"/>
       <c r="O188" s="10"/>
-      <c r="P188" s="10"/>
-      <c r="Q188" s="10"/>
-      <c r="R188" s="10"/>
     </row>
     <row r="189" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A189" s="10"/>
@@ -5845,9 +5260,6 @@
       <c r="M189" s="10"/>
       <c r="N189" s="10"/>
       <c r="O189" s="10"/>
-      <c r="P189" s="10"/>
-      <c r="Q189" s="10"/>
-      <c r="R189" s="10"/>
     </row>
     <row r="190" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A190" s="10"/>
@@ -5868,9 +5280,6 @@
       <c r="M190" s="10"/>
       <c r="N190" s="10"/>
       <c r="O190" s="10"/>
-      <c r="P190" s="10"/>
-      <c r="Q190" s="10"/>
-      <c r="R190" s="10"/>
     </row>
     <row r="191" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A191" s="10"/>
@@ -5891,9 +5300,6 @@
       <c r="M191" s="10"/>
       <c r="N191" s="10"/>
       <c r="O191" s="10"/>
-      <c r="P191" s="10"/>
-      <c r="Q191" s="10"/>
-      <c r="R191" s="10"/>
     </row>
     <row r="192" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A192" s="10"/>
@@ -5914,9 +5320,6 @@
       <c r="M192" s="10"/>
       <c r="N192" s="10"/>
       <c r="O192" s="10"/>
-      <c r="P192" s="10"/>
-      <c r="Q192" s="10"/>
-      <c r="R192" s="10"/>
     </row>
     <row r="193" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A193" s="10"/>
@@ -5937,9 +5340,6 @@
       <c r="M193" s="10"/>
       <c r="N193" s="10"/>
       <c r="O193" s="10"/>
-      <c r="P193" s="10"/>
-      <c r="Q193" s="10"/>
-      <c r="R193" s="10"/>
     </row>
     <row r="194" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A194" s="10"/>
@@ -5960,9 +5360,6 @@
       <c r="M194" s="10"/>
       <c r="N194" s="10"/>
       <c r="O194" s="10"/>
-      <c r="P194" s="10"/>
-      <c r="Q194" s="10"/>
-      <c r="R194" s="10"/>
     </row>
     <row r="195" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A195" s="10"/>
@@ -5983,9 +5380,6 @@
       <c r="M195" s="10"/>
       <c r="N195" s="10"/>
       <c r="O195" s="10"/>
-      <c r="P195" s="10"/>
-      <c r="Q195" s="10"/>
-      <c r="R195" s="10"/>
     </row>
     <row r="196" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A196" s="10"/>
@@ -6006,9 +5400,6 @@
       <c r="M196" s="10"/>
       <c r="N196" s="10"/>
       <c r="O196" s="10"/>
-      <c r="P196" s="10"/>
-      <c r="Q196" s="10"/>
-      <c r="R196" s="10"/>
     </row>
     <row r="197" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A197" s="10"/>
@@ -6029,9 +5420,6 @@
       <c r="M197" s="10"/>
       <c r="N197" s="10"/>
       <c r="O197" s="10"/>
-      <c r="P197" s="10"/>
-      <c r="Q197" s="10"/>
-      <c r="R197" s="10"/>
     </row>
     <row r="198" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A198" s="10"/>
@@ -6052,9 +5440,6 @@
       <c r="M198" s="10"/>
       <c r="N198" s="10"/>
       <c r="O198" s="10"/>
-      <c r="P198" s="10"/>
-      <c r="Q198" s="10"/>
-      <c r="R198" s="10"/>
     </row>
     <row r="199" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A199" s="10"/>
@@ -6075,9 +5460,6 @@
       <c r="M199" s="10"/>
       <c r="N199" s="10"/>
       <c r="O199" s="10"/>
-      <c r="P199" s="10"/>
-      <c r="Q199" s="10"/>
-      <c r="R199" s="10"/>
     </row>
     <row r="200" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A200" s="10"/>
@@ -6098,9 +5480,6 @@
       <c r="M200" s="10"/>
       <c r="N200" s="10"/>
       <c r="O200" s="10"/>
-      <c r="P200" s="10"/>
-      <c r="Q200" s="10"/>
-      <c r="R200" s="10"/>
     </row>
     <row r="201" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A201" s="10"/>
@@ -6121,9 +5500,6 @@
       <c r="M201" s="10"/>
       <c r="N201" s="10"/>
       <c r="O201" s="10"/>
-      <c r="P201" s="10"/>
-      <c r="Q201" s="10"/>
-      <c r="R201" s="10"/>
     </row>
     <row r="202" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A202" s="10"/>
@@ -6144,9 +5520,6 @@
       <c r="M202" s="10"/>
       <c r="N202" s="10"/>
       <c r="O202" s="10"/>
-      <c r="P202" s="10"/>
-      <c r="Q202" s="10"/>
-      <c r="R202" s="10"/>
     </row>
     <row r="203" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A203" s="10"/>
@@ -6167,9 +5540,6 @@
       <c r="M203" s="10"/>
       <c r="N203" s="10"/>
       <c r="O203" s="10"/>
-      <c r="P203" s="10"/>
-      <c r="Q203" s="10"/>
-      <c r="R203" s="10"/>
     </row>
     <row r="204" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A204" s="10"/>
@@ -6190,9 +5560,6 @@
       <c r="M204" s="10"/>
       <c r="N204" s="10"/>
       <c r="O204" s="10"/>
-      <c r="P204" s="10"/>
-      <c r="Q204" s="10"/>
-      <c r="R204" s="10"/>
     </row>
     <row r="205" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A205" s="10"/>
@@ -6213,9 +5580,6 @@
       <c r="M205" s="10"/>
       <c r="N205" s="10"/>
       <c r="O205" s="10"/>
-      <c r="P205" s="10"/>
-      <c r="Q205" s="10"/>
-      <c r="R205" s="10"/>
     </row>
     <row r="206" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A206" s="10"/>
@@ -6236,9 +5600,6 @@
       <c r="M206" s="10"/>
       <c r="N206" s="10"/>
       <c r="O206" s="10"/>
-      <c r="P206" s="10"/>
-      <c r="Q206" s="10"/>
-      <c r="R206" s="10"/>
     </row>
     <row r="207" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A207" s="10"/>
@@ -6259,9 +5620,6 @@
       <c r="M207" s="10"/>
       <c r="N207" s="10"/>
       <c r="O207" s="10"/>
-      <c r="P207" s="10"/>
-      <c r="Q207" s="10"/>
-      <c r="R207" s="10"/>
     </row>
     <row r="208" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A208" s="10"/>
@@ -6282,9 +5640,6 @@
       <c r="M208" s="10"/>
       <c r="N208" s="10"/>
       <c r="O208" s="10"/>
-      <c r="P208" s="10"/>
-      <c r="Q208" s="10"/>
-      <c r="R208" s="10"/>
     </row>
     <row r="209" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A209" s="10"/>
@@ -6305,9 +5660,6 @@
       <c r="M209" s="10"/>
       <c r="N209" s="10"/>
       <c r="O209" s="10"/>
-      <c r="P209" s="10"/>
-      <c r="Q209" s="10"/>
-      <c r="R209" s="10"/>
     </row>
     <row r="210" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A210" s="10"/>
@@ -6328,9 +5680,6 @@
       <c r="M210" s="10"/>
       <c r="N210" s="10"/>
       <c r="O210" s="10"/>
-      <c r="P210" s="10"/>
-      <c r="Q210" s="10"/>
-      <c r="R210" s="10"/>
     </row>
     <row r="211" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A211" s="10"/>
@@ -6351,9 +5700,6 @@
       <c r="M211" s="10"/>
       <c r="N211" s="10"/>
       <c r="O211" s="10"/>
-      <c r="P211" s="10"/>
-      <c r="Q211" s="10"/>
-      <c r="R211" s="10"/>
     </row>
     <row r="212" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A212" s="10"/>
@@ -6374,9 +5720,6 @@
       <c r="M212" s="10"/>
       <c r="N212" s="10"/>
       <c r="O212" s="10"/>
-      <c r="P212" s="10"/>
-      <c r="Q212" s="10"/>
-      <c r="R212" s="10"/>
     </row>
     <row r="213" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A213" s="10"/>
@@ -6397,9 +5740,6 @@
       <c r="M213" s="10"/>
       <c r="N213" s="10"/>
       <c r="O213" s="10"/>
-      <c r="P213" s="10"/>
-      <c r="Q213" s="10"/>
-      <c r="R213" s="10"/>
     </row>
     <row r="214" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A214" s="10"/>
@@ -6420,9 +5760,6 @@
       <c r="M214" s="10"/>
       <c r="N214" s="10"/>
       <c r="O214" s="10"/>
-      <c r="P214" s="10"/>
-      <c r="Q214" s="10"/>
-      <c r="R214" s="10"/>
     </row>
     <row r="215" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A215" s="10"/>
@@ -6443,9 +5780,6 @@
       <c r="M215" s="10"/>
       <c r="N215" s="10"/>
       <c r="O215" s="10"/>
-      <c r="P215" s="10"/>
-      <c r="Q215" s="10"/>
-      <c r="R215" s="10"/>
     </row>
     <row r="216" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A216" s="10"/>
@@ -6466,9 +5800,6 @@
       <c r="M216" s="10"/>
       <c r="N216" s="10"/>
       <c r="O216" s="10"/>
-      <c r="P216" s="10"/>
-      <c r="Q216" s="10"/>
-      <c r="R216" s="10"/>
     </row>
     <row r="217" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A217" s="10"/>
@@ -6489,9 +5820,6 @@
       <c r="M217" s="10"/>
       <c r="N217" s="10"/>
       <c r="O217" s="10"/>
-      <c r="P217" s="10"/>
-      <c r="Q217" s="10"/>
-      <c r="R217" s="10"/>
     </row>
     <row r="218" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A218" s="10"/>
@@ -6512,9 +5840,6 @@
       <c r="M218" s="10"/>
       <c r="N218" s="10"/>
       <c r="O218" s="10"/>
-      <c r="P218" s="10"/>
-      <c r="Q218" s="10"/>
-      <c r="R218" s="10"/>
     </row>
     <row r="219" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A219" s="10"/>
@@ -6535,9 +5860,6 @@
       <c r="M219" s="10"/>
       <c r="N219" s="10"/>
       <c r="O219" s="10"/>
-      <c r="P219" s="10"/>
-      <c r="Q219" s="10"/>
-      <c r="R219" s="10"/>
     </row>
     <row r="220" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A220" s="10"/>
@@ -6558,9 +5880,6 @@
       <c r="M220" s="10"/>
       <c r="N220" s="10"/>
       <c r="O220" s="10"/>
-      <c r="P220" s="10"/>
-      <c r="Q220" s="10"/>
-      <c r="R220" s="10"/>
     </row>
     <row r="221" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A221" s="10"/>
@@ -6581,9 +5900,6 @@
       <c r="M221" s="10"/>
       <c r="N221" s="10"/>
       <c r="O221" s="10"/>
-      <c r="P221" s="10"/>
-      <c r="Q221" s="10"/>
-      <c r="R221" s="10"/>
     </row>
     <row r="222" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A222" s="10"/>
@@ -6604,9 +5920,6 @@
       <c r="M222" s="10"/>
       <c r="N222" s="10"/>
       <c r="O222" s="10"/>
-      <c r="P222" s="10"/>
-      <c r="Q222" s="10"/>
-      <c r="R222" s="10"/>
     </row>
     <row r="223" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A223" s="10"/>
@@ -6627,9 +5940,6 @@
       <c r="M223" s="10"/>
       <c r="N223" s="10"/>
       <c r="O223" s="10"/>
-      <c r="P223" s="10"/>
-      <c r="Q223" s="10"/>
-      <c r="R223" s="10"/>
     </row>
     <row r="224" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A224" s="10"/>
@@ -6650,9 +5960,6 @@
       <c r="M224" s="10"/>
       <c r="N224" s="10"/>
       <c r="O224" s="10"/>
-      <c r="P224" s="10"/>
-      <c r="Q224" s="10"/>
-      <c r="R224" s="10"/>
     </row>
     <row r="225" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A225" s="10"/>
@@ -6673,9 +5980,6 @@
       <c r="M225" s="10"/>
       <c r="N225" s="10"/>
       <c r="O225" s="10"/>
-      <c r="P225" s="10"/>
-      <c r="Q225" s="10"/>
-      <c r="R225" s="10"/>
     </row>
     <row r="226" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A226" s="10"/>
@@ -6696,9 +6000,6 @@
       <c r="M226" s="10"/>
       <c r="N226" s="10"/>
       <c r="O226" s="10"/>
-      <c r="P226" s="10"/>
-      <c r="Q226" s="10"/>
-      <c r="R226" s="10"/>
     </row>
     <row r="227" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A227" s="10"/>
@@ -6719,9 +6020,6 @@
       <c r="M227" s="10"/>
       <c r="N227" s="10"/>
       <c r="O227" s="10"/>
-      <c r="P227" s="10"/>
-      <c r="Q227" s="10"/>
-      <c r="R227" s="10"/>
     </row>
     <row r="228" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A228" s="10"/>
@@ -6742,9 +6040,6 @@
       <c r="M228" s="10"/>
       <c r="N228" s="10"/>
       <c r="O228" s="10"/>
-      <c r="P228" s="10"/>
-      <c r="Q228" s="10"/>
-      <c r="R228" s="10"/>
     </row>
     <row r="229" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A229" s="10"/>
@@ -6765,9 +6060,6 @@
       <c r="M229" s="10"/>
       <c r="N229" s="10"/>
       <c r="O229" s="10"/>
-      <c r="P229" s="10"/>
-      <c r="Q229" s="10"/>
-      <c r="R229" s="10"/>
     </row>
     <row r="230" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A230" s="10"/>
@@ -6788,9 +6080,6 @@
       <c r="M230" s="10"/>
       <c r="N230" s="10"/>
       <c r="O230" s="10"/>
-      <c r="P230" s="10"/>
-      <c r="Q230" s="10"/>
-      <c r="R230" s="10"/>
     </row>
     <row r="231" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A231" s="10"/>
@@ -6811,9 +6100,6 @@
       <c r="M231" s="10"/>
       <c r="N231" s="10"/>
       <c r="O231" s="10"/>
-      <c r="P231" s="10"/>
-      <c r="Q231" s="10"/>
-      <c r="R231" s="10"/>
     </row>
     <row r="232" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A232" s="10"/>
@@ -6834,9 +6120,6 @@
       <c r="M232" s="10"/>
       <c r="N232" s="10"/>
       <c r="O232" s="10"/>
-      <c r="P232" s="10"/>
-      <c r="Q232" s="10"/>
-      <c r="R232" s="10"/>
     </row>
     <row r="233" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A233" s="10"/>
@@ -6857,9 +6140,6 @@
       <c r="M233" s="10"/>
       <c r="N233" s="10"/>
       <c r="O233" s="10"/>
-      <c r="P233" s="10"/>
-      <c r="Q233" s="10"/>
-      <c r="R233" s="10"/>
     </row>
     <row r="234" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A234" s="10"/>
@@ -6880,9 +6160,6 @@
       <c r="M234" s="10"/>
       <c r="N234" s="10"/>
       <c r="O234" s="10"/>
-      <c r="P234" s="10"/>
-      <c r="Q234" s="10"/>
-      <c r="R234" s="10"/>
     </row>
     <row r="235" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A235" s="10"/>
@@ -6903,9 +6180,6 @@
       <c r="M235" s="10"/>
       <c r="N235" s="10"/>
       <c r="O235" s="10"/>
-      <c r="P235" s="10"/>
-      <c r="Q235" s="10"/>
-      <c r="R235" s="10"/>
     </row>
     <row r="236" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A236" s="10"/>
@@ -6926,9 +6200,6 @@
       <c r="M236" s="10"/>
       <c r="N236" s="10"/>
       <c r="O236" s="10"/>
-      <c r="P236" s="10"/>
-      <c r="Q236" s="10"/>
-      <c r="R236" s="10"/>
     </row>
     <row r="237" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A237" s="10"/>
@@ -6949,9 +6220,6 @@
       <c r="M237" s="10"/>
       <c r="N237" s="10"/>
       <c r="O237" s="10"/>
-      <c r="P237" s="10"/>
-      <c r="Q237" s="10"/>
-      <c r="R237" s="10"/>
     </row>
     <row r="238" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A238" s="10"/>
@@ -6972,9 +6240,6 @@
       <c r="M238" s="10"/>
       <c r="N238" s="10"/>
       <c r="O238" s="10"/>
-      <c r="P238" s="10"/>
-      <c r="Q238" s="10"/>
-      <c r="R238" s="10"/>
     </row>
     <row r="239" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A239" s="10"/>
@@ -6995,9 +6260,6 @@
       <c r="M239" s="10"/>
       <c r="N239" s="10"/>
       <c r="O239" s="10"/>
-      <c r="P239" s="10"/>
-      <c r="Q239" s="10"/>
-      <c r="R239" s="10"/>
     </row>
     <row r="240" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A240" s="10"/>
@@ -7018,9 +6280,6 @@
       <c r="M240" s="10"/>
       <c r="N240" s="10"/>
       <c r="O240" s="10"/>
-      <c r="P240" s="10"/>
-      <c r="Q240" s="10"/>
-      <c r="R240" s="10"/>
     </row>
     <row r="241" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A241" s="10"/>
@@ -7041,9 +6300,6 @@
       <c r="M241" s="10"/>
       <c r="N241" s="10"/>
       <c r="O241" s="10"/>
-      <c r="P241" s="10"/>
-      <c r="Q241" s="10"/>
-      <c r="R241" s="10"/>
     </row>
     <row r="242" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A242" s="10"/>
@@ -7064,9 +6320,6 @@
       <c r="M242" s="10"/>
       <c r="N242" s="10"/>
       <c r="O242" s="10"/>
-      <c r="P242" s="10"/>
-      <c r="Q242" s="10"/>
-      <c r="R242" s="10"/>
     </row>
     <row r="243" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A243" s="10"/>
@@ -7087,9 +6340,6 @@
       <c r="M243" s="10"/>
       <c r="N243" s="10"/>
       <c r="O243" s="10"/>
-      <c r="P243" s="10"/>
-      <c r="Q243" s="10"/>
-      <c r="R243" s="10"/>
     </row>
     <row r="244" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A244" s="10"/>
@@ -7110,9 +6360,6 @@
       <c r="M244" s="10"/>
       <c r="N244" s="10"/>
       <c r="O244" s="10"/>
-      <c r="P244" s="10"/>
-      <c r="Q244" s="10"/>
-      <c r="R244" s="10"/>
     </row>
     <row r="245" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A245" s="10"/>
@@ -7133,9 +6380,6 @@
       <c r="M245" s="10"/>
       <c r="N245" s="10"/>
       <c r="O245" s="10"/>
-      <c r="P245" s="10"/>
-      <c r="Q245" s="10"/>
-      <c r="R245" s="10"/>
     </row>
     <row r="246" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A246" s="10"/>
@@ -7156,9 +6400,6 @@
       <c r="M246" s="10"/>
       <c r="N246" s="10"/>
       <c r="O246" s="10"/>
-      <c r="P246" s="10"/>
-      <c r="Q246" s="10"/>
-      <c r="R246" s="10"/>
     </row>
     <row r="247" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A247" s="10"/>
@@ -7179,9 +6420,6 @@
       <c r="M247" s="10"/>
       <c r="N247" s="10"/>
       <c r="O247" s="10"/>
-      <c r="P247" s="10"/>
-      <c r="Q247" s="10"/>
-      <c r="R247" s="10"/>
     </row>
     <row r="248" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A248" s="10"/>
@@ -7202,9 +6440,6 @@
       <c r="M248" s="10"/>
       <c r="N248" s="10"/>
       <c r="O248" s="10"/>
-      <c r="P248" s="10"/>
-      <c r="Q248" s="10"/>
-      <c r="R248" s="10"/>
     </row>
     <row r="249" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A249" s="10"/>
@@ -7225,9 +6460,6 @@
       <c r="M249" s="10"/>
       <c r="N249" s="10"/>
       <c r="O249" s="10"/>
-      <c r="P249" s="10"/>
-      <c r="Q249" s="10"/>
-      <c r="R249" s="10"/>
     </row>
     <row r="250" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A250" s="10"/>
@@ -7248,9 +6480,6 @@
       <c r="M250" s="10"/>
       <c r="N250" s="10"/>
       <c r="O250" s="10"/>
-      <c r="P250" s="10"/>
-      <c r="Q250" s="10"/>
-      <c r="R250" s="10"/>
     </row>
     <row r="251" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A251" s="10"/>
@@ -7271,9 +6500,6 @@
       <c r="M251" s="10"/>
       <c r="N251" s="10"/>
       <c r="O251" s="10"/>
-      <c r="P251" s="10"/>
-      <c r="Q251" s="10"/>
-      <c r="R251" s="10"/>
     </row>
     <row r="252" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A252" s="10"/>
@@ -7294,9 +6520,6 @@
       <c r="M252" s="10"/>
       <c r="N252" s="10"/>
       <c r="O252" s="10"/>
-      <c r="P252" s="10"/>
-      <c r="Q252" s="10"/>
-      <c r="R252" s="10"/>
     </row>
     <row r="253" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A253" s="10"/>
@@ -7317,9 +6540,6 @@
       <c r="M253" s="10"/>
       <c r="N253" s="10"/>
       <c r="O253" s="10"/>
-      <c r="P253" s="10"/>
-      <c r="Q253" s="10"/>
-      <c r="R253" s="10"/>
     </row>
     <row r="254" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A254" s="10"/>
@@ -7340,9 +6560,6 @@
       <c r="M254" s="10"/>
       <c r="N254" s="10"/>
       <c r="O254" s="10"/>
-      <c r="P254" s="10"/>
-      <c r="Q254" s="10"/>
-      <c r="R254" s="10"/>
     </row>
     <row r="255" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A255" s="10"/>
@@ -7363,9 +6580,6 @@
       <c r="M255" s="10"/>
       <c r="N255" s="10"/>
       <c r="O255" s="10"/>
-      <c r="P255" s="10"/>
-      <c r="Q255" s="10"/>
-      <c r="R255" s="10"/>
     </row>
     <row r="256" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A256" s="10"/>
@@ -7386,9 +6600,6 @@
       <c r="M256" s="10"/>
       <c r="N256" s="10"/>
       <c r="O256" s="10"/>
-      <c r="P256" s="10"/>
-      <c r="Q256" s="10"/>
-      <c r="R256" s="10"/>
     </row>
     <row r="257" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A257" s="10"/>
@@ -7409,9 +6620,6 @@
       <c r="M257" s="10"/>
       <c r="N257" s="10"/>
       <c r="O257" s="10"/>
-      <c r="P257" s="10"/>
-      <c r="Q257" s="10"/>
-      <c r="R257" s="10"/>
     </row>
     <row r="258" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A258" s="10"/>
@@ -7432,9 +6640,6 @@
       <c r="M258" s="10"/>
       <c r="N258" s="10"/>
       <c r="O258" s="10"/>
-      <c r="P258" s="10"/>
-      <c r="Q258" s="10"/>
-      <c r="R258" s="10"/>
     </row>
     <row r="259" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A259" s="10"/>
@@ -7455,9 +6660,6 @@
       <c r="M259" s="10"/>
       <c r="N259" s="10"/>
       <c r="O259" s="10"/>
-      <c r="P259" s="10"/>
-      <c r="Q259" s="10"/>
-      <c r="R259" s="10"/>
     </row>
     <row r="260" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A260" s="10"/>
@@ -7478,9 +6680,6 @@
       <c r="M260" s="10"/>
       <c r="N260" s="10"/>
       <c r="O260" s="10"/>
-      <c r="P260" s="10"/>
-      <c r="Q260" s="10"/>
-      <c r="R260" s="10"/>
     </row>
     <row r="261" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A261" s="10"/>
@@ -7501,9 +6700,6 @@
       <c r="M261" s="10"/>
       <c r="N261" s="10"/>
       <c r="O261" s="10"/>
-      <c r="P261" s="10"/>
-      <c r="Q261" s="10"/>
-      <c r="R261" s="10"/>
     </row>
     <row r="262" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A262" s="10"/>
@@ -7524,9 +6720,6 @@
       <c r="M262" s="10"/>
       <c r="N262" s="10"/>
       <c r="O262" s="10"/>
-      <c r="P262" s="10"/>
-      <c r="Q262" s="10"/>
-      <c r="R262" s="10"/>
     </row>
     <row r="263" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A263" s="10"/>
@@ -7547,9 +6740,6 @@
       <c r="M263" s="10"/>
       <c r="N263" s="10"/>
       <c r="O263" s="10"/>
-      <c r="P263" s="10"/>
-      <c r="Q263" s="10"/>
-      <c r="R263" s="10"/>
     </row>
     <row r="264" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A264" s="10"/>
@@ -7570,9 +6760,6 @@
       <c r="M264" s="10"/>
       <c r="N264" s="10"/>
       <c r="O264" s="10"/>
-      <c r="P264" s="10"/>
-      <c r="Q264" s="10"/>
-      <c r="R264" s="10"/>
     </row>
     <row r="265" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A265" s="10"/>
@@ -7593,9 +6780,6 @@
       <c r="M265" s="10"/>
       <c r="N265" s="10"/>
       <c r="O265" s="10"/>
-      <c r="P265" s="10"/>
-      <c r="Q265" s="10"/>
-      <c r="R265" s="10"/>
     </row>
     <row r="266" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A266" s="10"/>
@@ -7616,9 +6800,6 @@
       <c r="M266" s="10"/>
       <c r="N266" s="10"/>
       <c r="O266" s="10"/>
-      <c r="P266" s="10"/>
-      <c r="Q266" s="10"/>
-      <c r="R266" s="10"/>
     </row>
     <row r="267" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A267" s="10"/>
@@ -7639,9 +6820,6 @@
       <c r="M267" s="10"/>
       <c r="N267" s="10"/>
       <c r="O267" s="10"/>
-      <c r="P267" s="10"/>
-      <c r="Q267" s="10"/>
-      <c r="R267" s="10"/>
     </row>
     <row r="268" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A268" s="10"/>
@@ -7662,9 +6840,6 @@
       <c r="M268" s="10"/>
       <c r="N268" s="10"/>
       <c r="O268" s="10"/>
-      <c r="P268" s="10"/>
-      <c r="Q268" s="10"/>
-      <c r="R268" s="10"/>
     </row>
     <row r="269" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A269" s="10"/>
@@ -7685,9 +6860,6 @@
       <c r="M269" s="10"/>
       <c r="N269" s="10"/>
       <c r="O269" s="10"/>
-      <c r="P269" s="10"/>
-      <c r="Q269" s="10"/>
-      <c r="R269" s="10"/>
     </row>
     <row r="270" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A270" s="10"/>
@@ -7708,9 +6880,6 @@
       <c r="M270" s="10"/>
       <c r="N270" s="10"/>
       <c r="O270" s="10"/>
-      <c r="P270" s="10"/>
-      <c r="Q270" s="10"/>
-      <c r="R270" s="10"/>
     </row>
     <row r="271" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A271" s="10"/>
@@ -7731,9 +6900,6 @@
       <c r="M271" s="10"/>
       <c r="N271" s="10"/>
       <c r="O271" s="10"/>
-      <c r="P271" s="10"/>
-      <c r="Q271" s="10"/>
-      <c r="R271" s="10"/>
     </row>
     <row r="272" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A272" s="10"/>
@@ -7754,9 +6920,6 @@
       <c r="M272" s="10"/>
       <c r="N272" s="10"/>
       <c r="O272" s="10"/>
-      <c r="P272" s="10"/>
-      <c r="Q272" s="10"/>
-      <c r="R272" s="10"/>
     </row>
     <row r="273" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A273" s="10"/>
@@ -7777,9 +6940,6 @@
       <c r="M273" s="10"/>
       <c r="N273" s="10"/>
       <c r="O273" s="10"/>
-      <c r="P273" s="10"/>
-      <c r="Q273" s="10"/>
-      <c r="R273" s="10"/>
     </row>
     <row r="274" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A274" s="10"/>
@@ -7800,9 +6960,6 @@
       <c r="M274" s="10"/>
       <c r="N274" s="10"/>
       <c r="O274" s="10"/>
-      <c r="P274" s="10"/>
-      <c r="Q274" s="10"/>
-      <c r="R274" s="10"/>
     </row>
     <row r="275" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A275" s="10"/>
@@ -7823,9 +6980,6 @@
       <c r="M275" s="10"/>
       <c r="N275" s="10"/>
       <c r="O275" s="10"/>
-      <c r="P275" s="10"/>
-      <c r="Q275" s="10"/>
-      <c r="R275" s="10"/>
     </row>
     <row r="276" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A276" s="10"/>
@@ -7846,9 +7000,6 @@
       <c r="M276" s="10"/>
       <c r="N276" s="10"/>
       <c r="O276" s="10"/>
-      <c r="P276" s="10"/>
-      <c r="Q276" s="10"/>
-      <c r="R276" s="10"/>
     </row>
     <row r="277" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A277" s="10"/>
@@ -7869,9 +7020,6 @@
       <c r="M277" s="10"/>
       <c r="N277" s="10"/>
       <c r="O277" s="10"/>
-      <c r="P277" s="10"/>
-      <c r="Q277" s="10"/>
-      <c r="R277" s="10"/>
     </row>
     <row r="278" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A278" s="10"/>
@@ -7892,9 +7040,6 @@
       <c r="M278" s="10"/>
       <c r="N278" s="10"/>
       <c r="O278" s="10"/>
-      <c r="P278" s="10"/>
-      <c r="Q278" s="10"/>
-      <c r="R278" s="10"/>
     </row>
     <row r="279" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A279" s="10"/>
@@ -7915,9 +7060,6 @@
       <c r="M279" s="10"/>
       <c r="N279" s="10"/>
       <c r="O279" s="10"/>
-      <c r="P279" s="10"/>
-      <c r="Q279" s="10"/>
-      <c r="R279" s="10"/>
     </row>
     <row r="280" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A280" s="10"/>
@@ -7938,9 +7080,6 @@
       <c r="M280" s="10"/>
       <c r="N280" s="10"/>
       <c r="O280" s="10"/>
-      <c r="P280" s="10"/>
-      <c r="Q280" s="10"/>
-      <c r="R280" s="10"/>
     </row>
     <row r="281" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A281" s="10"/>
@@ -7961,9 +7100,6 @@
       <c r="M281" s="10"/>
       <c r="N281" s="10"/>
       <c r="O281" s="10"/>
-      <c r="P281" s="10"/>
-      <c r="Q281" s="10"/>
-      <c r="R281" s="10"/>
     </row>
     <row r="282" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A282" s="10"/>
@@ -7984,9 +7120,6 @@
       <c r="M282" s="10"/>
       <c r="N282" s="10"/>
       <c r="O282" s="10"/>
-      <c r="P282" s="10"/>
-      <c r="Q282" s="10"/>
-      <c r="R282" s="10"/>
     </row>
     <row r="283" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A283" s="10"/>
@@ -8007,9 +7140,6 @@
       <c r="M283" s="10"/>
       <c r="N283" s="10"/>
       <c r="O283" s="10"/>
-      <c r="P283" s="10"/>
-      <c r="Q283" s="10"/>
-      <c r="R283" s="10"/>
     </row>
     <row r="284" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A284" s="10"/>
@@ -8030,9 +7160,6 @@
       <c r="M284" s="10"/>
       <c r="N284" s="10"/>
       <c r="O284" s="10"/>
-      <c r="P284" s="10"/>
-      <c r="Q284" s="10"/>
-      <c r="R284" s="10"/>
     </row>
     <row r="285" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A285" s="10"/>
@@ -8053,9 +7180,6 @@
       <c r="M285" s="10"/>
       <c r="N285" s="10"/>
       <c r="O285" s="10"/>
-      <c r="P285" s="10"/>
-      <c r="Q285" s="10"/>
-      <c r="R285" s="10"/>
     </row>
     <row r="286" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A286" s="10"/>
@@ -8076,9 +7200,6 @@
       <c r="M286" s="10"/>
       <c r="N286" s="10"/>
       <c r="O286" s="10"/>
-      <c r="P286" s="10"/>
-      <c r="Q286" s="10"/>
-      <c r="R286" s="10"/>
     </row>
     <row r="287" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A287" s="10"/>
@@ -8099,9 +7220,6 @@
       <c r="M287" s="10"/>
       <c r="N287" s="10"/>
       <c r="O287" s="10"/>
-      <c r="P287" s="10"/>
-      <c r="Q287" s="10"/>
-      <c r="R287" s="10"/>
     </row>
     <row r="288" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A288" s="10"/>
@@ -8122,9 +7240,6 @@
       <c r="M288" s="10"/>
       <c r="N288" s="10"/>
       <c r="O288" s="10"/>
-      <c r="P288" s="10"/>
-      <c r="Q288" s="10"/>
-      <c r="R288" s="10"/>
     </row>
     <row r="289" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A289" s="10"/>
@@ -8145,9 +7260,6 @@
       <c r="M289" s="10"/>
       <c r="N289" s="10"/>
       <c r="O289" s="10"/>
-      <c r="P289" s="10"/>
-      <c r="Q289" s="10"/>
-      <c r="R289" s="10"/>
     </row>
     <row r="290" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A290" s="10"/>
@@ -8168,9 +7280,6 @@
       <c r="M290" s="10"/>
       <c r="N290" s="10"/>
       <c r="O290" s="10"/>
-      <c r="P290" s="10"/>
-      <c r="Q290" s="10"/>
-      <c r="R290" s="10"/>
     </row>
     <row r="291" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A291" s="10"/>
@@ -8191,9 +7300,6 @@
       <c r="M291" s="10"/>
       <c r="N291" s="10"/>
       <c r="O291" s="10"/>
-      <c r="P291" s="10"/>
-      <c r="Q291" s="10"/>
-      <c r="R291" s="10"/>
     </row>
     <row r="292" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A292" s="10"/>
@@ -8214,9 +7320,6 @@
       <c r="M292" s="10"/>
       <c r="N292" s="10"/>
       <c r="O292" s="10"/>
-      <c r="P292" s="10"/>
-      <c r="Q292" s="10"/>
-      <c r="R292" s="10"/>
     </row>
     <row r="293" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A293" s="10"/>
@@ -8237,9 +7340,6 @@
       <c r="M293" s="10"/>
       <c r="N293" s="10"/>
       <c r="O293" s="10"/>
-      <c r="P293" s="10"/>
-      <c r="Q293" s="10"/>
-      <c r="R293" s="10"/>
     </row>
     <row r="294" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A294" s="10"/>
@@ -8260,9 +7360,6 @@
       <c r="M294" s="10"/>
       <c r="N294" s="10"/>
       <c r="O294" s="10"/>
-      <c r="P294" s="10"/>
-      <c r="Q294" s="10"/>
-      <c r="R294" s="10"/>
     </row>
     <row r="295" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A295" s="10"/>
@@ -8283,9 +7380,6 @@
       <c r="M295" s="10"/>
       <c r="N295" s="10"/>
       <c r="O295" s="10"/>
-      <c r="P295" s="10"/>
-      <c r="Q295" s="10"/>
-      <c r="R295" s="10"/>
     </row>
     <row r="296" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A296" s="10"/>
@@ -8306,9 +7400,6 @@
       <c r="M296" s="10"/>
       <c r="N296" s="10"/>
       <c r="O296" s="10"/>
-      <c r="P296" s="10"/>
-      <c r="Q296" s="10"/>
-      <c r="R296" s="10"/>
     </row>
     <row r="297" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A297" s="10"/>
@@ -8329,9 +7420,6 @@
       <c r="M297" s="10"/>
       <c r="N297" s="10"/>
       <c r="O297" s="10"/>
-      <c r="P297" s="10"/>
-      <c r="Q297" s="10"/>
-      <c r="R297" s="10"/>
     </row>
     <row r="298" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A298" s="10"/>
@@ -8352,9 +7440,6 @@
       <c r="M298" s="10"/>
       <c r="N298" s="10"/>
       <c r="O298" s="10"/>
-      <c r="P298" s="10"/>
-      <c r="Q298" s="10"/>
-      <c r="R298" s="10"/>
     </row>
     <row r="299" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A299" s="10"/>
@@ -8375,9 +7460,6 @@
       <c r="M299" s="10"/>
       <c r="N299" s="10"/>
       <c r="O299" s="10"/>
-      <c r="P299" s="10"/>
-      <c r="Q299" s="10"/>
-      <c r="R299" s="10"/>
     </row>
     <row r="300" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A300" s="10"/>
@@ -8398,9 +7480,6 @@
       <c r="M300" s="10"/>
       <c r="N300" s="10"/>
       <c r="O300" s="10"/>
-      <c r="P300" s="10"/>
-      <c r="Q300" s="10"/>
-      <c r="R300" s="10"/>
     </row>
     <row r="301" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A301" s="10"/>
@@ -8421,9 +7500,6 @@
       <c r="M301" s="10"/>
       <c r="N301" s="10"/>
       <c r="O301" s="10"/>
-      <c r="P301" s="10"/>
-      <c r="Q301" s="10"/>
-      <c r="R301" s="10"/>
     </row>
     <row r="302" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A302" s="10"/>
@@ -8444,9 +7520,6 @@
       <c r="M302" s="10"/>
       <c r="N302" s="10"/>
       <c r="O302" s="10"/>
-      <c r="P302" s="10"/>
-      <c r="Q302" s="10"/>
-      <c r="R302" s="10"/>
     </row>
     <row r="303" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A303" s="10"/>
@@ -8467,9 +7540,6 @@
       <c r="M303" s="10"/>
       <c r="N303" s="10"/>
       <c r="O303" s="10"/>
-      <c r="P303" s="10"/>
-      <c r="Q303" s="10"/>
-      <c r="R303" s="10"/>
     </row>
     <row r="304" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A304" s="10"/>
@@ -8490,16 +7560,13 @@
       <c r="M304" s="10"/>
       <c r="N304" s="10"/>
       <c r="O304" s="10"/>
-      <c r="P304" s="10"/>
-      <c r="Q304" s="10"/>
-      <c r="R304" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:R1"/>
     <mergeCell ref="A2:R2"/>
   </mergeCells>
-  <dataValidations count="8">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" sqref="C10:C304">
       <formula1>"Mobilizasyon,Kolon Montajı,Kiriş Montajı,Aşık Montajı,Panel Montajı,Elektrik DC,Elektrik AC,Elektrik OG,Köşk Trafo,Topraklama,ENH,Devreye Alma,Evrak Süreci,Satın Alma,Mekanik"</formula1>
     </dataValidation>
@@ -8511,18 +7578,6 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="I5:I304">
       <formula1>"beklemede,devam_ediyor,tamamlandi,askida,iptal"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="P10:P304">
-      <formula1>"Evet,Hayır"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="P5:P304">
-      <formula1>"Evet,Hayır"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="R10:R304">
-      <formula1>"Evet,Hayır"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="R5:R304">
-      <formula1>"Evet,Hayır"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8543,7 +7598,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -8551,7 +7606,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -8559,139 +7614,139 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D4" s="9"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B5" s="12">
         <v>10</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D5" s="12"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B6" s="12">
         <v>10</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D6" s="12"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B7" s="12">
         <v>10</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D7" s="12"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B8" s="12">
         <v>20</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D8" s="12"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B9" s="12">
         <v>10</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D9" s="12"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B10" s="12">
         <v>10</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D10" s="12"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B11" s="12">
         <v>10</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D11" s="12"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B12" s="12">
         <v>5</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D12" s="12"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B13" s="12">
         <v>5</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D13" s="12"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B14" s="12">
         <v>10</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="D14" s="12"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B15" s="13">
         <f>SUM(B5:B14)</f>
@@ -8700,7 +7755,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -8734,7 +7789,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8748,7 +7803,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8762,34 +7817,34 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>82</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>87</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>11</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -14197,7 +13252,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" sqref="D10:E304">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
@@ -14209,6 +13264,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="H5:H304">
       <formula1>"açık,azaltıldı,kabul_edildi,kapatıldı"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="J10:J304">
+      <formula1>"İş Kalemi,Satın Alma,Diğer"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="J5:J304">
       <formula1>"İş Kalemi,Satın Alma,Diğer"</formula1>
@@ -14238,7 +13296,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -14247,7 +13305,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -14256,7 +13314,7 @@
     </row>
     <row r="3" ht="28.05" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B3"/>
       <c r="C3"/>
@@ -14265,41 +13323,41 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="7:11" x14ac:dyDescent="0.25">
       <c r="G4" s="17" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="H4"/>
       <c r="J4" s="17" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="K4"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -14309,13 +13367,13 @@
       <c r="D6" s="22"/>
       <c r="E6" s="20"/>
       <c r="G6" s="23" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="H6" s="24" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="J6" s="25" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="K6" s="26">
         <f>SUMIF($A$6:$A$305,"panel",$C$6:$C$305)</f>
@@ -14329,13 +13387,13 @@
       <c r="D7" s="22"/>
       <c r="E7" s="20"/>
       <c r="G7" s="27" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H7" s="28" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="J7" s="29" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="K7" s="30">
         <f>SUMIF($A$6:$A$305,"inverter",$C$6:$C$305)</f>
@@ -14349,13 +13407,13 @@
       <c r="D8" s="22"/>
       <c r="E8" s="20"/>
       <c r="G8" s="23" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="H8" s="24" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J8" s="25" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="K8" s="26">
         <f>SUMIF($A$6:$A$305,"mekanik",$C$6:$C$305)</f>
@@ -14369,13 +13427,13 @@
       <c r="D9" s="22"/>
       <c r="E9" s="20"/>
       <c r="G9" s="27" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="K9" s="30">
         <f>SUMIF($A$6:$A$305,"elektrik_dc",$C$6:$C$305)</f>
@@ -14389,13 +13447,13 @@
       <c r="D10" s="22"/>
       <c r="E10" s="20"/>
       <c r="G10" s="23" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="J10" s="25" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="K10" s="26">
         <f>SUMIF($A$6:$A$305,"elektrik_ac",$C$6:$C$305)</f>
@@ -14409,13 +13467,13 @@
       <c r="D11" s="22"/>
       <c r="E11" s="20"/>
       <c r="G11" s="27" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="H11" s="28" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="J11" s="29" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="K11" s="30">
         <f>SUMIF($A$6:$A$305,"elektrik_og",$C$6:$C$305)</f>
@@ -14429,13 +13487,13 @@
       <c r="D12" s="22"/>
       <c r="E12" s="20"/>
       <c r="G12" s="23" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="H12" s="24" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="J12" s="25" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="K12" s="26">
         <f>SUMIF($A$6:$A$305,"enh",$C$6:$C$305)</f>
@@ -14449,13 +13507,13 @@
       <c r="D13" s="22"/>
       <c r="E13" s="20"/>
       <c r="G13" s="27" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="H13" s="28" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="J13" s="29" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="K13" s="30">
         <f>SUMIF($A$6:$A$305,"altyapi",$C$6:$C$305)</f>
@@ -14469,13 +13527,13 @@
       <c r="D14" s="22"/>
       <c r="E14" s="20"/>
       <c r="G14" s="23" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="H14" s="24" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="J14" s="25" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="K14" s="26">
         <f>SUMIF($A$6:$A$305,"iscilik",$C$6:$C$305)</f>
@@ -14489,13 +13547,13 @@
       <c r="D15" s="22"/>
       <c r="E15" s="20"/>
       <c r="G15" s="27" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="H15" s="28" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="J15" s="29" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="K15" s="30">
         <f>SUMIF($A$6:$A$305,"izin",$C$6:$C$305)</f>
@@ -14509,13 +13567,13 @@
       <c r="D16" s="22"/>
       <c r="E16" s="20"/>
       <c r="G16" s="23" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="H16" s="24" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="J16" s="25" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="K16" s="26">
         <f>SUMIF($A$6:$A$305,"denetim",$C$6:$C$305)</f>
@@ -14529,13 +13587,13 @@
       <c r="D17" s="22"/>
       <c r="E17" s="20"/>
       <c r="G17" s="27" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="H17" s="28" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="J17" s="29" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="K17" s="30">
         <f>SUMIF($A$6:$A$305,"diger",$C$6:$C$305)</f>
@@ -14549,7 +13607,7 @@
       <c r="D18" s="22"/>
       <c r="E18" s="20"/>
       <c r="J18" s="31" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="K18" s="32">
         <f>SUM(K6:K17)</f>
@@ -14570,7 +13628,7 @@
       <c r="D20" s="22"/>
       <c r="E20" s="20"/>
       <c r="J20" s="33" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="K20" s="34">
         <f>COUNTIF($A$6:$A$305,"&lt;&gt;")</f>
@@ -16619,7 +15677,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -16634,7 +15692,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -16649,37 +15707,37 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C4" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="I4" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="J4" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>132</v>
-      </c>
       <c r="K4" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -20618,7 +19676,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -20626,108 +19684,112 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
       <c r="D2"/>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="3:3" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="57" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" ht="28.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C7" s="35" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="C9" s="35" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>152</v>
-      </c>
-    </row>
+        <v>147</v>
+      </c>
+    </row>
+    <row r="11" spans="3:3" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="3:3" x14ac:dyDescent="0.25"/>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C13" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C14" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C15" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C16" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>